<commit_message>
Simplifica clientes con nombre comercial, sectores, Plus Code y logo
</commit_message>
<xml_diff>
--- a/public/templates/Plantilla-clientes-EMSA.xlsx
+++ b/public/templates/Plantilla-clientes-EMSA.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="1" r:id="Ra902f06a81fe4a0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cliente" sheetId="2" r:id="R6494ac2f4c394fda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacto" sheetId="3" r:id="Rfa792370bf4c4024"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sede" sheetId="4" r:id="R22cfaf7538d845c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="1" r:id="Rb299d5d676c24288"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cliente" sheetId="2" r:id="R0a270c17b0ed4200"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacto" sheetId="3" r:id="Ra75275d312ee4c75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sede" sheetId="4" r:id="R825c57e463c44a38"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="@"/>
-    <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -122,7 +121,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -150,20 +149,14 @@
     <x:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -409,637 +402,637 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
-      <x:c r="A1" s="17"/>
-      <x:c r="B1" s="17"/>
-      <x:c r="C1" s="17"/>
-      <x:c r="D1" s="17"/>
-      <x:c r="E1" s="17"/>
+      <x:c r="A1" s="15"/>
+      <x:c r="B1" s="15"/>
+      <x:c r="C1" s="15"/>
+      <x:c r="D1" s="15"/>
+      <x:c r="E1" s="15"/>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
-      <x:c r="A2" s="18" t="str">
+      <x:c r="A2" s="16" t="str">
         <x:v>Clientes EMSA</x:v>
       </x:c>
-      <x:c r="B2" s="17"/>
-      <x:c r="C2" s="17"/>
-      <x:c r="D2" s="17"/>
-      <x:c r="E2" s="17"/>
+      <x:c r="B2" s="15"/>
+      <x:c r="C2" s="15"/>
+      <x:c r="D2" s="15"/>
+      <x:c r="E2" s="15"/>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
-      <x:c r="A3" s="19"/>
-      <x:c r="B3" s="19"/>
-      <x:c r="C3" s="19"/>
-      <x:c r="D3" s="19"/>
-      <x:c r="E3" s="19"/>
+      <x:c r="A3" s="17"/>
+      <x:c r="B3" s="17"/>
+      <x:c r="C3" s="17"/>
+      <x:c r="D3" s="17"/>
+      <x:c r="E3" s="17"/>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
-      <x:c r="A4" s="17"/>
-      <x:c r="B4" s="17"/>
-      <x:c r="C4" s="17"/>
-      <x:c r="D4" s="17"/>
-      <x:c r="E4" s="17"/>
+      <x:c r="A4" s="15"/>
+      <x:c r="B4" s="15"/>
+      <x:c r="C4" s="15"/>
+      <x:c r="D4" s="15"/>
+      <x:c r="E4" s="15"/>
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
-      <x:c r="A5" s="20" t="str">
+      <x:c r="A5" s="18" t="str">
         <x:v>Para empezar</x:v>
       </x:c>
-      <x:c r="B5" s="17" t="str">
+      <x:c r="B5" s="15" t="str">
         <x:v>Llena Cliente desde la fila 2. Usa una fila por empresa.</x:v>
       </x:c>
-      <x:c r="C5" s="17"/>
-      <x:c r="D5" s="17"/>
-      <x:c r="E5" s="17"/>
+      <x:c r="C5" s="15"/>
+      <x:c r="D5" s="15"/>
+      <x:c r="E5" s="15"/>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
-      <x:c r="A6" s="20" t="str">
+      <x:c r="A6" s="18" t="str">
         <x:v>Datos mínimos</x:v>
       </x:c>
-      <x:c r="B6" s="17" t="str">
-        <x:v>referencia_cliente, nombre y estado. Las columnas ámbar son obligatorias.</x:v>
-      </x:c>
-      <x:c r="C6" s="17"/>
-      <x:c r="D6" s="17"/>
-      <x:c r="E6" s="17"/>
+      <x:c r="B6" s="15" t="str">
+        <x:v>nombre (razón social) y estado. Las columnas ámbar son obligatorias. El código CLI es automático.</x:v>
+      </x:c>
+      <x:c r="C6" s="15"/>
+      <x:c r="D6" s="15"/>
+      <x:c r="E6" s="15"/>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
-      <x:c r="A7" s="20" t="str">
+      <x:c r="A7" s="18" t="str">
         <x:v>Referencia</x:v>
       </x:c>
-      <x:c r="B7" s="17" t="str">
-        <x:v>Asigna C001, C002, etc. Repite la referencia en los contactos y sedes de esa empresa.</x:v>
-      </x:c>
-      <x:c r="C7" s="17"/>
-      <x:c r="D7" s="17"/>
-      <x:c r="E7" s="17"/>
+      <x:c r="B7" s="15" t="str">
+        <x:v>Solo para vincular contactos/sedes: asigna C001, C002, etc. y repítelo en esas hojas.</x:v>
+      </x:c>
+      <x:c r="C7" s="15"/>
+      <x:c r="D7" s="15"/>
+      <x:c r="E7" s="15"/>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
-      <x:c r="A8" s="20" t="str">
+      <x:c r="A8" s="18" t="str">
         <x:v>Contactos y sedes</x:v>
       </x:c>
-      <x:c r="B8" s="17" t="str">
+      <x:c r="B8" s="15" t="str">
         <x:v>Una fila por contacto o sede. Puedes tener varios por empresa; no repitas la empresa en Cliente.</x:v>
       </x:c>
-      <x:c r="C8" s="17"/>
-      <x:c r="D8" s="17"/>
-      <x:c r="E8" s="17"/>
+      <x:c r="C8" s="15"/>
+      <x:c r="D8" s="15"/>
+      <x:c r="E8" s="15"/>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
-      <x:c r="A9" s="20" t="str">
+      <x:c r="A9" s="18" t="str">
         <x:v>Datos faltantes</x:v>
       </x:c>
-      <x:c r="B9" s="17" t="str">
+      <x:c r="B9" s="15" t="str">
         <x:v>Deja vacíos los datos desconocidos. No uses cero para representar información faltante.</x:v>
       </x:c>
-      <x:c r="C9" s="17"/>
-      <x:c r="D9" s="17"/>
-      <x:c r="E9" s="17"/>
+      <x:c r="C9" s="15"/>
+      <x:c r="D9" s="15"/>
+      <x:c r="E9" s="15"/>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
-      <x:c r="A10" s="20" t="str">
+      <x:c r="A10" s="18" t="str">
         <x:v>Formato</x:v>
       </x:c>
-      <x:c r="B10" s="17" t="str">
+      <x:c r="B10" s="15" t="str">
         <x:v>Conserva nombres de hojas y encabezados. NIT, referencias y teléfonos se guardan como texto.</x:v>
       </x:c>
-      <x:c r="C10" s="17"/>
-      <x:c r="D10" s="17"/>
-      <x:c r="E10" s="17"/>
+      <x:c r="C10" s="15"/>
+      <x:c r="D10" s="15"/>
+      <x:c r="E10" s="15"/>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
-      <x:c r="A11" s="20" t="str">
+      <x:c r="A11" s="18" t="str">
         <x:v>Cómo importarlo</x:v>
       </x:c>
-      <x:c r="B11" s="17" t="str">
+      <x:c r="B11" s="15" t="str">
         <x:v>En Administrador: Clientes &gt; Importar clientes. Selecciona el Excel y revisa la vista previa.</x:v>
       </x:c>
-      <x:c r="C11" s="17"/>
-      <x:c r="D11" s="17"/>
-      <x:c r="E11" s="17"/>
+      <x:c r="C11" s="15"/>
+      <x:c r="D11" s="15"/>
+      <x:c r="E11" s="15"/>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
-      <x:c r="A12" s="20" t="str">
+      <x:c r="A12" s="18" t="str">
         <x:v>Antes de guardar</x:v>
       </x:c>
-      <x:c r="B12" s="17" t="str">
+      <x:c r="B12" s="15" t="str">
         <x:v>Corrige errores y confirma la importación. Clientes, contactos y sedes se guardan juntos.</x:v>
       </x:c>
-      <x:c r="C12" s="17"/>
-      <x:c r="D12" s="17"/>
-      <x:c r="E12" s="17"/>
+      <x:c r="C12" s="15"/>
+      <x:c r="D12" s="15"/>
+      <x:c r="E12" s="15"/>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
-      <x:c r="A13" s="20" t="str">
-        <x:v>Alcance</x:v>
-      </x:c>
-      <x:c r="B13" s="17" t="str">
-        <x:v>Campos propuestos según tu documento maestro. Contratos, SLA y equipos se preparan por separado.</x:v>
-      </x:c>
-      <x:c r="C13" s="17"/>
-      <x:c r="D13" s="17"/>
-      <x:c r="E13" s="17"/>
+      <x:c r="A13" s="18" t="str">
+        <x:v>Logo</x:v>
+      </x:c>
+      <x:c r="B13" s="15" t="str">
+        <x:v>El logo se sube desde la ficha del cliente en la web. Esta plantilla no incluye imágenes.</x:v>
+      </x:c>
+      <x:c r="C13" s="15"/>
+      <x:c r="D13" s="15"/>
+      <x:c r="E13" s="15"/>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
-      <x:c r="A14" s="20" t="str">
+      <x:c r="A14" s="18" t="str">
         <x:v>Ejemplos</x:v>
       </x:c>
-      <x:c r="B14" s="17" t="str">
+      <x:c r="B14" s="15" t="str">
         <x:v>Los ejemplos de abajo son ficticios. Las tres hojas de captura están vacías.</x:v>
       </x:c>
-      <x:c r="C14" s="17"/>
-      <x:c r="D14" s="17"/>
-      <x:c r="E14" s="17"/>
+      <x:c r="C14" s="15"/>
+      <x:c r="D14" s="15"/>
+      <x:c r="E14" s="15"/>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
-      <x:c r="A15" s="17"/>
-      <x:c r="B15" s="17"/>
-      <x:c r="C15" s="17"/>
-      <x:c r="D15" s="17"/>
-      <x:c r="E15" s="17"/>
+      <x:c r="A15" s="15"/>
+      <x:c r="B15" s="15"/>
+      <x:c r="C15" s="15"/>
+      <x:c r="D15" s="15"/>
+      <x:c r="E15" s="15"/>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="23" t="str">
+      <x:c r="A16" s="21" t="str">
         <x:v>Hoja</x:v>
       </x:c>
-      <x:c r="B16" s="23" t="str">
+      <x:c r="B16" s="21" t="str">
         <x:v>Campo</x:v>
       </x:c>
-      <x:c r="C16" s="23" t="str">
+      <x:c r="C16" s="21" t="str">
         <x:v>Necesario</x:v>
       </x:c>
-      <x:c r="D16" s="23" t="str">
+      <x:c r="D16" s="21" t="str">
         <x:v>Qué registrar</x:v>
       </x:c>
-      <x:c r="E16" s="23" t="str">
+      <x:c r="E16" s="21" t="str">
         <x:v>Ejemplo ficticio</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="29" customHeight="1">
-      <x:c r="A17" s="24" t="str">
+      <x:c r="A17" s="22" t="str">
         <x:v>Cliente</x:v>
       </x:c>
-      <x:c r="B17" s="24" t="str">
+      <x:c r="B17" s="22" t="str">
         <x:v>referencia_cliente</x:v>
       </x:c>
-      <x:c r="C17" s="26" t="str">
+      <x:c r="C17" s="22" t="str">
+        <x:v>Si agregas vínculos</x:v>
+      </x:c>
+      <x:c r="D17" s="22" t="str">
+        <x:v>Referencia para vincular contactos/sedes; no es el código CLI automático.</x:v>
+      </x:c>
+      <x:c r="E17" s="22" t="str">
+        <x:v>C001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="29" customHeight="1">
+      <x:c r="A18" s="15" t="str">
+        <x:v>Cliente</x:v>
+      </x:c>
+      <x:c r="B18" s="15" t="str">
+        <x:v>nombre</x:v>
+      </x:c>
+      <x:c r="C18" s="24" t="str">
         <x:v>Obligatorio</x:v>
       </x:c>
-      <x:c r="D17" s="24" t="str">
-        <x:v>Referencia única en este archivo; no es el ID automático del portal.</x:v>
-      </x:c>
-      <x:c r="E17" s="24" t="str">
+      <x:c r="D18" s="15" t="str">
+        <x:v>Razón social de la empresa.</x:v>
+      </x:c>
+      <x:c r="E18" s="15" t="str">
+        <x:v>Empresa de ejemplo, S.A.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="29" customHeight="1">
+      <x:c r="A19" s="22" t="str">
+        <x:v>Cliente</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>nombre_comercial</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>Recomendado</x:v>
+      </x:c>
+      <x:c r="D19" s="22" t="str">
+        <x:v>Nombre comercial o nombre por el que se conoce a la empresa.</x:v>
+      </x:c>
+      <x:c r="E19" s="22" t="str">
+        <x:v>Comercial de ejemplo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="29" customHeight="1">
+      <x:c r="A20" s="15" t="str">
+        <x:v>Cliente</x:v>
+      </x:c>
+      <x:c r="B20" s="15" t="str">
+        <x:v>estado</x:v>
+      </x:c>
+      <x:c r="C20" s="24" t="str">
+        <x:v>Obligatorio</x:v>
+      </x:c>
+      <x:c r="D20" s="15" t="str">
+        <x:v>Selecciona Activo, Prospecto o Inactivo.</x:v>
+      </x:c>
+      <x:c r="E20" s="15" t="str">
+        <x:v>Activo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="29" customHeight="1">
+      <x:c r="A21" s="22" t="str">
+        <x:v>Cliente</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>nit</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>Recomendado</x:v>
+      </x:c>
+      <x:c r="D21" s="22" t="str">
+        <x:v>NIT tal como aparece en tus registros; conservar guiones y dígitos.</x:v>
+      </x:c>
+      <x:c r="E21" s="22" t="str">
+        <x:v>Texto del NIT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="29" customHeight="1">
+      <x:c r="A22" s="15" t="str">
+        <x:v>Cliente</x:v>
+      </x:c>
+      <x:c r="B22" s="15" t="str">
+        <x:v>sector</x:v>
+      </x:c>
+      <x:c r="C22" s="15" t="str">
+        <x:v>Opcional</x:v>
+      </x:c>
+      <x:c r="D22" s="15" t="str">
+        <x:v>Selecciona la actividad o giro de la empresa.</x:v>
+      </x:c>
+      <x:c r="E22" s="15" t="str">
+        <x:v>Comercio y distribución</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="29" customHeight="1">
+      <x:c r="A23" s="22" t="str">
+        <x:v>Cliente</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>ubicacion</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="str">
+        <x:v>Recomendado</x:v>
+      </x:c>
+      <x:c r="D23" s="22" t="str">
+        <x:v>Municipio o ubicación principal para identificar al cliente.</x:v>
+      </x:c>
+      <x:c r="E23" s="22" t="str">
+        <x:v>Villa Nueva</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="29" customHeight="1">
+      <x:c r="A24" s="15" t="str">
+        <x:v>Cliente</x:v>
+      </x:c>
+      <x:c r="B24" s="15" t="str">
+        <x:v>plus_code</x:v>
+      </x:c>
+      <x:c r="C24" s="15" t="str">
+        <x:v>Opcional</x:v>
+      </x:c>
+      <x:c r="D24" s="15" t="str">
+        <x:v>Copia el Plus Code completo con su localidad desde Google Maps.</x:v>
+      </x:c>
+      <x:c r="E24" s="15" t="str">
+        <x:v>Código y localidad</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="29" customHeight="1">
+      <x:c r="A25" s="22" t="str">
+        <x:v>Cliente</x:v>
+      </x:c>
+      <x:c r="B25" s="22" t="str">
+        <x:v>direccion_fiscal</x:v>
+      </x:c>
+      <x:c r="C25" s="22" t="str">
+        <x:v>Recomendado</x:v>
+      </x:c>
+      <x:c r="D25" s="22" t="str">
+        <x:v>Dirección utilizada en la documentación de facturación.</x:v>
+      </x:c>
+      <x:c r="E25" s="22" t="str">
+        <x:v>Dirección fiscal de ejemplo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="29" customHeight="1">
+      <x:c r="A26" s="15" t="str">
+        <x:v>Cliente</x:v>
+      </x:c>
+      <x:c r="B26" s="15" t="str">
+        <x:v>notas_operativas</x:v>
+      </x:c>
+      <x:c r="C26" s="15" t="str">
+        <x:v>Opcional</x:v>
+      </x:c>
+      <x:c r="D26" s="15" t="str">
+        <x:v>Instrucciones generales relevantes para atender a la empresa.</x:v>
+      </x:c>
+      <x:c r="E26" s="15" t="str">
+        <x:v>Coordinar visitas con recepción.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="29" customHeight="1">
+      <x:c r="A27" s="22" t="str">
+        <x:v>Contacto</x:v>
+      </x:c>
+      <x:c r="B27" s="22" t="str">
+        <x:v>referencia_cliente</x:v>
+      </x:c>
+      <x:c r="C27" s="22" t="str">
+        <x:v>Al agregar contacto</x:v>
+      </x:c>
+      <x:c r="D27" s="22" t="str">
+        <x:v>La misma referencia que existe en la hoja Cliente.</x:v>
+      </x:c>
+      <x:c r="E27" s="22" t="str">
         <x:v>C001</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="29" customHeight="1">
-      <x:c r="A18" s="17" t="str">
-        <x:v>Cliente</x:v>
-      </x:c>
-      <x:c r="B18" s="17" t="str">
+    <x:row r="28" ht="29" customHeight="1">
+      <x:c r="A28" s="15" t="str">
+        <x:v>Contacto</x:v>
+      </x:c>
+      <x:c r="B28" s="15" t="str">
         <x:v>nombre</x:v>
       </x:c>
-      <x:c r="C18" s="26" t="str">
-        <x:v>Obligatorio</x:v>
-      </x:c>
-      <x:c r="D18" s="17" t="str">
-        <x:v>Nombre de la empresa o razón social.</x:v>
-      </x:c>
-      <x:c r="E18" s="17" t="str">
-        <x:v>Empresa de ejemplo, S.A.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="29" customHeight="1">
-      <x:c r="A19" s="24" t="str">
-        <x:v>Cliente</x:v>
-      </x:c>
-      <x:c r="B19" s="24" t="str">
-        <x:v>estado</x:v>
-      </x:c>
-      <x:c r="C19" s="26" t="str">
-        <x:v>Obligatorio</x:v>
-      </x:c>
-      <x:c r="D19" s="24" t="str">
-        <x:v>Selecciona Activo, Prospecto o Inactivo.</x:v>
-      </x:c>
-      <x:c r="E19" s="24" t="str">
-        <x:v>Activo</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="29" customHeight="1">
-      <x:c r="A20" s="17" t="str">
-        <x:v>Cliente</x:v>
-      </x:c>
-      <x:c r="B20" s="17" t="str">
-        <x:v>nit</x:v>
-      </x:c>
-      <x:c r="C20" s="17" t="str">
+      <x:c r="C28" s="15" t="str">
+        <x:v>Al agregar contacto</x:v>
+      </x:c>
+      <x:c r="D28" s="15" t="str">
+        <x:v>Nombre de la persona de contacto.</x:v>
+      </x:c>
+      <x:c r="E28" s="15" t="str">
+        <x:v>Persona de ejemplo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="29" customHeight="1">
+      <x:c r="A29" s="22" t="str">
+        <x:v>Contacto</x:v>
+      </x:c>
+      <x:c r="B29" s="22" t="str">
+        <x:v>cargo</x:v>
+      </x:c>
+      <x:c r="C29" s="22" t="str">
+        <x:v>Opcional</x:v>
+      </x:c>
+      <x:c r="D29" s="22" t="str">
+        <x:v>Responsabilidad o área.</x:v>
+      </x:c>
+      <x:c r="E29" s="22" t="str">
+        <x:v>Mantenimiento</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="29" customHeight="1">
+      <x:c r="A30" s="15" t="str">
+        <x:v>Contacto</x:v>
+      </x:c>
+      <x:c r="B30" s="15" t="str">
+        <x:v>telefono</x:v>
+      </x:c>
+      <x:c r="C30" s="15" t="str">
         <x:v>Recomendado</x:v>
       </x:c>
-      <x:c r="D20" s="17" t="str">
-        <x:v>NIT tal como aparece en tus registros; conservar guiones y dígitos.</x:v>
-      </x:c>
-      <x:c r="E20" s="17" t="str">
-        <x:v>Texto del NIT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="29" customHeight="1">
-      <x:c r="A21" s="24" t="str">
-        <x:v>Cliente</x:v>
-      </x:c>
-      <x:c r="B21" s="24" t="str">
-        <x:v>sector</x:v>
-      </x:c>
-      <x:c r="C21" s="24" t="str">
+      <x:c r="D30" s="15" t="str">
+        <x:v>Número con código de país cuando corresponda; almacenar como texto.</x:v>
+      </x:c>
+      <x:c r="E30" s="15" t="str">
+        <x:v>+502 0000 0000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="29" customHeight="1">
+      <x:c r="A31" s="22" t="str">
+        <x:v>Contacto</x:v>
+      </x:c>
+      <x:c r="B31" s="22" t="str">
+        <x:v>correo</x:v>
+      </x:c>
+      <x:c r="C31" s="22" t="str">
+        <x:v>Recomendado</x:v>
+      </x:c>
+      <x:c r="D31" s="22" t="str">
+        <x:v>Correo de contacto; procura tener teléfono o correo.</x:v>
+      </x:c>
+      <x:c r="E31" s="22" t="str">
+        <x:v>contacto@example.com</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="29" customHeight="1">
+      <x:c r="A32" s="15" t="str">
+        <x:v>Contacto</x:v>
+      </x:c>
+      <x:c r="B32" s="15" t="str">
+        <x:v>principal</x:v>
+      </x:c>
+      <x:c r="C32" s="15" t="str">
         <x:v>Opcional</x:v>
       </x:c>
-      <x:c r="D21" s="24" t="str">
-        <x:v>Actividad o giro de la empresa.</x:v>
-      </x:c>
-      <x:c r="E21" s="24" t="str">
-        <x:v>Distribución</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="29" customHeight="1">
-      <x:c r="A22" s="17" t="str">
-        <x:v>Cliente</x:v>
-      </x:c>
-      <x:c r="B22" s="17" t="str">
-        <x:v>ubicacion</x:v>
-      </x:c>
-      <x:c r="C22" s="17" t="str">
+      <x:c r="D32" s="15" t="str">
+        <x:v>Marca Sí para identificar el contacto principal de la empresa.</x:v>
+      </x:c>
+      <x:c r="E32" s="15" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="29" customHeight="1">
+      <x:c r="A33" s="22" t="str">
+        <x:v>Sede</x:v>
+      </x:c>
+      <x:c r="B33" s="22" t="str">
+        <x:v>referencia_cliente</x:v>
+      </x:c>
+      <x:c r="C33" s="22" t="str">
+        <x:v>Al agregar sede</x:v>
+      </x:c>
+      <x:c r="D33" s="22" t="str">
+        <x:v>La misma referencia que existe en la hoja Cliente.</x:v>
+      </x:c>
+      <x:c r="E33" s="22" t="str">
+        <x:v>C001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="29" customHeight="1">
+      <x:c r="A34" s="15" t="str">
+        <x:v>Sede</x:v>
+      </x:c>
+      <x:c r="B34" s="15" t="str">
+        <x:v>nombre</x:v>
+      </x:c>
+      <x:c r="C34" s="15" t="str">
+        <x:v>Al agregar sede</x:v>
+      </x:c>
+      <x:c r="D34" s="15" t="str">
+        <x:v>Nombre de la sede, bodega o planta.</x:v>
+      </x:c>
+      <x:c r="E34" s="15" t="str">
+        <x:v>Bodega central</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="29" customHeight="1">
+      <x:c r="A35" s="22" t="str">
+        <x:v>Sede</x:v>
+      </x:c>
+      <x:c r="B35" s="22" t="str">
+        <x:v>direccion</x:v>
+      </x:c>
+      <x:c r="C35" s="22" t="str">
         <x:v>Recomendado</x:v>
       </x:c>
-      <x:c r="D22" s="17" t="str">
-        <x:v>Municipio o ubicación principal para identificar al cliente.</x:v>
-      </x:c>
-      <x:c r="E22" s="17" t="str">
+      <x:c r="D35" s="22" t="str">
+        <x:v>Dirección física y referencias útiles para llegar.</x:v>
+      </x:c>
+      <x:c r="E35" s="22" t="str">
+        <x:v>Dirección de ejemplo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="29" customHeight="1">
+      <x:c r="A36" s="15" t="str">
+        <x:v>Sede</x:v>
+      </x:c>
+      <x:c r="B36" s="15" t="str">
+        <x:v>municipio</x:v>
+      </x:c>
+      <x:c r="C36" s="15" t="str">
+        <x:v>Recomendado</x:v>
+      </x:c>
+      <x:c r="D36" s="15" t="str">
+        <x:v>Municipio en el que se encuentra la sede.</x:v>
+      </x:c>
+      <x:c r="E36" s="15" t="str">
         <x:v>Villa Nueva</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="29" customHeight="1">
-      <x:c r="A23" s="24" t="str">
-        <x:v>Cliente</x:v>
-      </x:c>
-      <x:c r="B23" s="24" t="str">
-        <x:v>direccion_fiscal</x:v>
-      </x:c>
-      <x:c r="C23" s="24" t="str">
+    <x:row r="37" ht="29" customHeight="1">
+      <x:c r="A37" s="22" t="str">
+        <x:v>Sede</x:v>
+      </x:c>
+      <x:c r="B37" s="22" t="str">
+        <x:v>departamento</x:v>
+      </x:c>
+      <x:c r="C37" s="22" t="str">
         <x:v>Recomendado</x:v>
       </x:c>
-      <x:c r="D23" s="24" t="str">
-        <x:v>Dirección utilizada en la documentación de facturación.</x:v>
-      </x:c>
-      <x:c r="E23" s="24" t="str">
-        <x:v>Dirección fiscal de ejemplo</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="29" customHeight="1">
-      <x:c r="A24" s="17" t="str">
-        <x:v>Cliente</x:v>
-      </x:c>
-      <x:c r="B24" s="17" t="str">
-        <x:v>dia_facturacion</x:v>
-      </x:c>
-      <x:c r="C24" s="17" t="str">
-        <x:v>Opcional</x:v>
-      </x:c>
-      <x:c r="D24" s="17" t="str">
-        <x:v>Día habitual del mes, del 1 al 31. Si varía, explícalo en notas.</x:v>
-      </x:c>
-      <x:c r="E24" s="17" t="str">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="29" customHeight="1">
-      <x:c r="A25" s="24" t="str">
-        <x:v>Cliente</x:v>
-      </x:c>
-      <x:c r="B25" s="24" t="str">
-        <x:v>reporte_mensual_horas</x:v>
-      </x:c>
-      <x:c r="C25" s="24" t="str">
-        <x:v>Opcional</x:v>
-      </x:c>
-      <x:c r="D25" s="24" t="str">
-        <x:v>Indica Sí o No; deja vacío si aún no se ha acordado.</x:v>
-      </x:c>
-      <x:c r="E25" s="24" t="str">
-        <x:v>Sí</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="29" customHeight="1">
-      <x:c r="A26" s="17" t="str">
-        <x:v>Cliente</x:v>
-      </x:c>
-      <x:c r="B26" s="17" t="str">
-        <x:v>notas_operativas</x:v>
-      </x:c>
-      <x:c r="C26" s="17" t="str">
-        <x:v>Opcional</x:v>
-      </x:c>
-      <x:c r="D26" s="17" t="str">
-        <x:v>Instrucciones generales relevantes para atender a la empresa.</x:v>
-      </x:c>
-      <x:c r="E26" s="17" t="str">
-        <x:v>Coordinar visitas con recepción.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="29" customHeight="1">
-      <x:c r="A27" s="24" t="str">
-        <x:v>Contacto</x:v>
-      </x:c>
-      <x:c r="B27" s="24" t="str">
-        <x:v>referencia_cliente</x:v>
-      </x:c>
-      <x:c r="C27" s="24" t="str">
-        <x:v>Al agregar contacto</x:v>
-      </x:c>
-      <x:c r="D27" s="24" t="str">
-        <x:v>La misma referencia que existe en la hoja Cliente.</x:v>
-      </x:c>
-      <x:c r="E27" s="24" t="str">
-        <x:v>C001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="29" customHeight="1">
-      <x:c r="A28" s="17" t="str">
-        <x:v>Contacto</x:v>
-      </x:c>
-      <x:c r="B28" s="17" t="str">
-        <x:v>nombre</x:v>
-      </x:c>
-      <x:c r="C28" s="17" t="str">
-        <x:v>Al agregar contacto</x:v>
-      </x:c>
-      <x:c r="D28" s="17" t="str">
-        <x:v>Nombre de la persona de contacto.</x:v>
-      </x:c>
-      <x:c r="E28" s="17" t="str">
-        <x:v>Persona de ejemplo</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="29" customHeight="1">
-      <x:c r="A29" s="24" t="str">
-        <x:v>Contacto</x:v>
-      </x:c>
-      <x:c r="B29" s="24" t="str">
-        <x:v>cargo</x:v>
-      </x:c>
-      <x:c r="C29" s="24" t="str">
-        <x:v>Opcional</x:v>
-      </x:c>
-      <x:c r="D29" s="24" t="str">
-        <x:v>Responsabilidad o área.</x:v>
-      </x:c>
-      <x:c r="E29" s="24" t="str">
-        <x:v>Mantenimiento</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="29" customHeight="1">
-      <x:c r="A30" s="17" t="str">
-        <x:v>Contacto</x:v>
-      </x:c>
-      <x:c r="B30" s="17" t="str">
-        <x:v>telefono</x:v>
-      </x:c>
-      <x:c r="C30" s="17" t="str">
+      <x:c r="D37" s="22" t="str">
+        <x:v>Departamento en el que se encuentra la sede.</x:v>
+      </x:c>
+      <x:c r="E37" s="22" t="str">
+        <x:v>Guatemala</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="29" customHeight="1">
+      <x:c r="A38" s="15" t="str">
+        <x:v>Sede</x:v>
+      </x:c>
+      <x:c r="B38" s="15" t="str">
+        <x:v>horario_atencion</x:v>
+      </x:c>
+      <x:c r="C38" s="15" t="str">
         <x:v>Recomendado</x:v>
       </x:c>
-      <x:c r="D30" s="17" t="str">
-        <x:v>Número con código de país cuando corresponda; almacenar como texto.</x:v>
-      </x:c>
-      <x:c r="E30" s="17" t="str">
-        <x:v>+502 0000 0000</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="29" customHeight="1">
-      <x:c r="A31" s="24" t="str">
-        <x:v>Contacto</x:v>
-      </x:c>
-      <x:c r="B31" s="24" t="str">
-        <x:v>correo</x:v>
-      </x:c>
-      <x:c r="C31" s="24" t="str">
+      <x:c r="D38" s="15" t="str">
+        <x:v>Días y horarios permitidos para servicios o visitas.</x:v>
+      </x:c>
+      <x:c r="E38" s="15" t="str">
+        <x:v>Lunes a viernes de 8:00 a 17:00</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="29" customHeight="1">
+      <x:c r="A39" s="22" t="str">
+        <x:v>Sede</x:v>
+      </x:c>
+      <x:c r="B39" s="22" t="str">
+        <x:v>autoriza_ingreso</x:v>
+      </x:c>
+      <x:c r="C39" s="22" t="str">
         <x:v>Recomendado</x:v>
       </x:c>
-      <x:c r="D31" s="24" t="str">
-        <x:v>Correo de contacto; procura tener teléfono o correo.</x:v>
-      </x:c>
-      <x:c r="E31" s="24" t="str">
-        <x:v>contacto@example.com</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="29" customHeight="1">
-      <x:c r="A32" s="17" t="str">
-        <x:v>Contacto</x:v>
-      </x:c>
-      <x:c r="B32" s="17" t="str">
-        <x:v>principal</x:v>
-      </x:c>
-      <x:c r="C32" s="17" t="str">
-        <x:v>Opcional</x:v>
-      </x:c>
-      <x:c r="D32" s="17" t="str">
-        <x:v>Marca Sí para identificar el contacto principal de la empresa.</x:v>
-      </x:c>
-      <x:c r="E32" s="17" t="str">
-        <x:v>Sí</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="29" customHeight="1">
-      <x:c r="A33" s="24" t="str">
-        <x:v>Sede</x:v>
-      </x:c>
-      <x:c r="B33" s="24" t="str">
-        <x:v>referencia_cliente</x:v>
-      </x:c>
-      <x:c r="C33" s="24" t="str">
-        <x:v>Al agregar sede</x:v>
-      </x:c>
-      <x:c r="D33" s="24" t="str">
-        <x:v>La misma referencia que existe en la hoja Cliente.</x:v>
-      </x:c>
-      <x:c r="E33" s="24" t="str">
-        <x:v>C001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="29" customHeight="1">
-      <x:c r="A34" s="17" t="str">
-        <x:v>Sede</x:v>
-      </x:c>
-      <x:c r="B34" s="17" t="str">
-        <x:v>nombre</x:v>
-      </x:c>
-      <x:c r="C34" s="17" t="str">
-        <x:v>Al agregar sede</x:v>
-      </x:c>
-      <x:c r="D34" s="17" t="str">
-        <x:v>Nombre de la sede, bodega o planta.</x:v>
-      </x:c>
-      <x:c r="E34" s="17" t="str">
-        <x:v>Bodega central</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="29" customHeight="1">
-      <x:c r="A35" s="24" t="str">
-        <x:v>Sede</x:v>
-      </x:c>
-      <x:c r="B35" s="24" t="str">
-        <x:v>direccion</x:v>
-      </x:c>
-      <x:c r="C35" s="24" t="str">
-        <x:v>Recomendado</x:v>
-      </x:c>
-      <x:c r="D35" s="24" t="str">
-        <x:v>Dirección física y referencias útiles para llegar.</x:v>
-      </x:c>
-      <x:c r="E35" s="24" t="str">
-        <x:v>Dirección de ejemplo</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="29" customHeight="1">
-      <x:c r="A36" s="17" t="str">
-        <x:v>Sede</x:v>
-      </x:c>
-      <x:c r="B36" s="17" t="str">
-        <x:v>municipio</x:v>
-      </x:c>
-      <x:c r="C36" s="17" t="str">
-        <x:v>Recomendado</x:v>
-      </x:c>
-      <x:c r="D36" s="17" t="str">
-        <x:v>Municipio en el que se encuentra la sede.</x:v>
-      </x:c>
-      <x:c r="E36" s="17" t="str">
-        <x:v>Villa Nueva</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="29" customHeight="1">
-      <x:c r="A37" s="24" t="str">
-        <x:v>Sede</x:v>
-      </x:c>
-      <x:c r="B37" s="24" t="str">
-        <x:v>departamento</x:v>
-      </x:c>
-      <x:c r="C37" s="24" t="str">
-        <x:v>Recomendado</x:v>
-      </x:c>
-      <x:c r="D37" s="24" t="str">
-        <x:v>Departamento en el que se encuentra la sede.</x:v>
-      </x:c>
-      <x:c r="E37" s="24" t="str">
-        <x:v>Guatemala</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="29" customHeight="1">
-      <x:c r="A38" s="17" t="str">
-        <x:v>Sede</x:v>
-      </x:c>
-      <x:c r="B38" s="17" t="str">
-        <x:v>horario_atencion</x:v>
-      </x:c>
-      <x:c r="C38" s="17" t="str">
-        <x:v>Recomendado</x:v>
-      </x:c>
-      <x:c r="D38" s="17" t="str">
-        <x:v>Días y horarios permitidos para servicios o visitas.</x:v>
-      </x:c>
-      <x:c r="E38" s="17" t="str">
-        <x:v>Lunes a viernes de 8:00 a 17:00</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="29" customHeight="1">
-      <x:c r="A39" s="24" t="str">
-        <x:v>Sede</x:v>
-      </x:c>
-      <x:c r="B39" s="24" t="str">
-        <x:v>autoriza_ingreso</x:v>
-      </x:c>
-      <x:c r="C39" s="24" t="str">
-        <x:v>Recomendado</x:v>
-      </x:c>
-      <x:c r="D39" s="24" t="str">
+      <x:c r="D39" s="22" t="str">
         <x:v>Persona o cargo que autoriza la entrada del técnico.</x:v>
       </x:c>
-      <x:c r="E39" s="24" t="str">
+      <x:c r="E39" s="22" t="str">
         <x:v>Jefatura de mantenimiento</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="25" customHeight="1">
-      <x:c r="A40" s="17"/>
-      <x:c r="B40" s="17"/>
-      <x:c r="C40" s="17"/>
-      <x:c r="D40" s="17"/>
-      <x:c r="E40" s="17"/>
+      <x:c r="A40" s="15"/>
+      <x:c r="B40" s="15"/>
+      <x:c r="C40" s="15"/>
+      <x:c r="D40" s="15"/>
+      <x:c r="E40" s="15"/>
     </x:row>
     <x:row r="41" ht="25" customHeight="1">
-      <x:c r="A41" s="17"/>
-      <x:c r="B41" s="17"/>
-      <x:c r="C41" s="17"/>
-      <x:c r="D41" s="17"/>
-      <x:c r="E41" s="17"/>
+      <x:c r="A41" s="15"/>
+      <x:c r="B41" s="15"/>
+      <x:c r="C41" s="15"/>
+      <x:c r="D41" s="15"/>
+      <x:c r="E41" s="15"/>
     </x:row>
     <x:row r="42" ht="25" customHeight="1">
-      <x:c r="A42" s="17" t="str">
+      <x:c r="A42" s="15" t="str">
         <x:v>Preparación</x:v>
       </x:c>
-      <x:c r="B42" s="17" t="str">
+      <x:c r="B42" s="15" t="str">
         <x:v>100 filas disponibles por hoja. Agrega más filas si las necesitas.</x:v>
       </x:c>
-      <x:c r="C42" s="17"/>
-      <x:c r="D42" s="17"/>
-      <x:c r="E42" s="17"/>
+      <x:c r="C42" s="15"/>
+      <x:c r="D42" s="15"/>
+      <x:c r="E42" s="15"/>
     </x:row>
     <x:row r="43" ht="25" customHeight="1">
-      <x:c r="A43" s="17"/>
-      <x:c r="B43" s="17"/>
-      <x:c r="C43" s="17"/>
-      <x:c r="D43" s="17"/>
-      <x:c r="E43" s="17"/>
+      <x:c r="A43" s="15"/>
+      <x:c r="B43" s="15"/>
+      <x:c r="C43" s="15"/>
+      <x:c r="D43" s="15"/>
+      <x:c r="E43" s="15"/>
     </x:row>
     <x:row r="44" ht="25" customHeight="1">
-      <x:c r="A44" s="17" t="str">
+      <x:c r="A44" s="15" t="str">
         <x:v>Fuente</x:v>
       </x:c>
-      <x:c r="B44" s="17" t="str">
-        <x:v>Documento maestro Portal EM, sección Clientes y contratos, proporcionado por el usuario.</x:v>
-      </x:c>
-      <x:c r="C44" s="17"/>
-      <x:c r="D44" s="17"/>
-      <x:c r="E44" s="17"/>
+      <x:c r="B44" s="15" t="str">
+        <x:v>Requisitos de clientes de Portal EM y ajustes solicitados el 07/10/2026.</x:v>
+      </x:c>
+      <x:c r="C44" s="15"/>
+      <x:c r="D44" s="15"/>
+      <x:c r="E44" s="15"/>
     </x:row>
     <x:row r="45" ht="25" customHeight="1">
-      <x:c r="A45" s="17"/>
-      <x:c r="B45" s="17"/>
-      <x:c r="C45" s="17"/>
-      <x:c r="D45" s="17"/>
-      <x:c r="E45" s="17"/>
+      <x:c r="A45" s="15"/>
+      <x:c r="B45" s="15"/>
+      <x:c r="C45" s="15"/>
+      <x:c r="D45" s="15"/>
+      <x:c r="E45" s="15"/>
     </x:row>
     <x:row r="46" ht="25" customHeight="1">
-      <x:c r="A46" s="17"/>
-      <x:c r="B46" s="17"/>
-      <x:c r="C46" s="17"/>
-      <x:c r="D46" s="17"/>
-      <x:c r="E46" s="17"/>
+      <x:c r="A46" s="15"/>
+      <x:c r="B46" s="15"/>
+      <x:c r="C46" s="15"/>
+      <x:c r="D46" s="15"/>
+      <x:c r="E46" s="15"/>
     </x:row>
     <x:row r="47" ht="25" customHeight="1">
-      <x:c r="A47" s="17"/>
-      <x:c r="B47" s="17"/>
-      <x:c r="C47" s="17"/>
-      <x:c r="D47" s="17"/>
-      <x:c r="E47" s="17"/>
+      <x:c r="A47" s="15"/>
+      <x:c r="B47" s="15"/>
+      <x:c r="C47" s="15"/>
+      <x:c r="D47" s="15"/>
+      <x:c r="E47" s="15"/>
     </x:row>
     <x:row r="48" ht="25" customHeight="1">
-      <x:c r="A48" s="17"/>
-      <x:c r="B48" s="17"/>
-      <x:c r="C48" s="17"/>
-      <x:c r="D48" s="17"/>
-      <x:c r="E48" s="17"/>
+      <x:c r="A48" s="15"/>
+      <x:c r="B48" s="15"/>
+      <x:c r="C48" s="15"/>
+      <x:c r="D48" s="15"/>
+      <x:c r="E48" s="15"/>
     </x:row>
     <x:row r="49" ht="25" customHeight="1">
-      <x:c r="A49" s="17"/>
-      <x:c r="B49" s="17"/>
-      <x:c r="C49" s="17"/>
-      <x:c r="D49" s="17"/>
-      <x:c r="E49" s="17"/>
+      <x:c r="A49" s="15"/>
+      <x:c r="B49" s="15"/>
+      <x:c r="C49" s="15"/>
+      <x:c r="D49" s="15"/>
+      <x:c r="E49" s="15"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1055,1259 +1048,1255 @@
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="40" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="50" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="21" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="27" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="50" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="55" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="35" customHeight="1">
-      <x:c r="A1" s="11" t="str">
+      <x:c r="A1" s="7" t="str">
         <x:v>referencia_cliente</x:v>
       </x:c>
-      <x:c r="B1" s="13" t="str">
+      <x:c r="B1" s="11" t="str">
         <x:v>nombre</x:v>
       </x:c>
-      <x:c r="C1" s="13" t="str">
+      <x:c r="C1" s="8" t="str">
+        <x:v>nombre_comercial</x:v>
+      </x:c>
+      <x:c r="D1" s="11" t="str">
         <x:v>estado</x:v>
       </x:c>
-      <x:c r="D1" s="8" t="str">
+      <x:c r="E1" s="8" t="str">
         <x:v>nit</x:v>
       </x:c>
-      <x:c r="E1" s="8" t="str">
+      <x:c r="F1" s="8" t="str">
         <x:v>sector</x:v>
       </x:c>
-      <x:c r="F1" s="8" t="str">
+      <x:c r="G1" s="8" t="str">
         <x:v>ubicacion</x:v>
       </x:c>
-      <x:c r="G1" s="8" t="str">
+      <x:c r="H1" s="8" t="str">
+        <x:v>plus_code</x:v>
+      </x:c>
+      <x:c r="I1" s="8" t="str">
         <x:v>direccion_fiscal</x:v>
-      </x:c>
-      <x:c r="H1" s="8" t="str">
-        <x:v>dia_facturacion</x:v>
-      </x:c>
-      <x:c r="I1" s="8" t="str">
-        <x:v>reporte_mensual_horas</x:v>
       </x:c>
       <x:c r="J1" s="9" t="str">
         <x:v>notas_operativas</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
-      <x:c r="A2" s="12"/>
+      <x:c r="A2" s="10"/>
       <x:c r="B2" s="12"/>
-      <x:c r="C2" s="12"/>
-      <x:c r="D2" s="10"/>
+      <x:c r="C2" s="10"/>
+      <x:c r="D2" s="12"/>
       <x:c r="E2" s="10"/>
       <x:c r="F2" s="10"/>
       <x:c r="G2" s="10"/>
-      <x:c r="H2" s="14"/>
+      <x:c r="H2" s="10"/>
       <x:c r="I2" s="10"/>
       <x:c r="J2" s="10"/>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
-      <x:c r="A3" s="12"/>
+      <x:c r="A3" s="3"/>
       <x:c r="B3" s="12"/>
-      <x:c r="C3" s="12"/>
-      <x:c r="D3" s="3"/>
+      <x:c r="C3" s="3"/>
+      <x:c r="D3" s="12"/>
       <x:c r="E3" s="3"/>
       <x:c r="F3" s="3"/>
       <x:c r="G3" s="3"/>
-      <x:c r="H3" s="15"/>
+      <x:c r="H3" s="3"/>
       <x:c r="I3" s="3"/>
       <x:c r="J3" s="3"/>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
-      <x:c r="A4" s="12"/>
+      <x:c r="A4" s="10"/>
       <x:c r="B4" s="12"/>
-      <x:c r="C4" s="12"/>
-      <x:c r="D4" s="10"/>
+      <x:c r="C4" s="10"/>
+      <x:c r="D4" s="12"/>
       <x:c r="E4" s="10"/>
       <x:c r="F4" s="10"/>
       <x:c r="G4" s="10"/>
-      <x:c r="H4" s="14"/>
+      <x:c r="H4" s="10"/>
       <x:c r="I4" s="10"/>
       <x:c r="J4" s="10"/>
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
-      <x:c r="A5" s="12"/>
+      <x:c r="A5" s="3"/>
       <x:c r="B5" s="12"/>
-      <x:c r="C5" s="12"/>
-      <x:c r="D5" s="3"/>
+      <x:c r="C5" s="3"/>
+      <x:c r="D5" s="12"/>
       <x:c r="E5" s="3"/>
       <x:c r="F5" s="3"/>
       <x:c r="G5" s="3"/>
-      <x:c r="H5" s="15"/>
+      <x:c r="H5" s="3"/>
       <x:c r="I5" s="3"/>
       <x:c r="J5" s="3"/>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
-      <x:c r="A6" s="12"/>
+      <x:c r="A6" s="10"/>
       <x:c r="B6" s="12"/>
-      <x:c r="C6" s="12"/>
-      <x:c r="D6" s="10"/>
+      <x:c r="C6" s="10"/>
+      <x:c r="D6" s="12"/>
       <x:c r="E6" s="10"/>
       <x:c r="F6" s="10"/>
       <x:c r="G6" s="10"/>
-      <x:c r="H6" s="14"/>
+      <x:c r="H6" s="10"/>
       <x:c r="I6" s="10"/>
       <x:c r="J6" s="10"/>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
-      <x:c r="A7" s="12"/>
+      <x:c r="A7" s="3"/>
       <x:c r="B7" s="12"/>
-      <x:c r="C7" s="12"/>
-      <x:c r="D7" s="3"/>
+      <x:c r="C7" s="3"/>
+      <x:c r="D7" s="12"/>
       <x:c r="E7" s="3"/>
       <x:c r="F7" s="3"/>
       <x:c r="G7" s="3"/>
-      <x:c r="H7" s="15"/>
+      <x:c r="H7" s="3"/>
       <x:c r="I7" s="3"/>
       <x:c r="J7" s="3"/>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
-      <x:c r="A8" s="12"/>
+      <x:c r="A8" s="10"/>
       <x:c r="B8" s="12"/>
-      <x:c r="C8" s="12"/>
-      <x:c r="D8" s="10"/>
+      <x:c r="C8" s="10"/>
+      <x:c r="D8" s="12"/>
       <x:c r="E8" s="10"/>
       <x:c r="F8" s="10"/>
       <x:c r="G8" s="10"/>
-      <x:c r="H8" s="14"/>
+      <x:c r="H8" s="10"/>
       <x:c r="I8" s="10"/>
       <x:c r="J8" s="10"/>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
-      <x:c r="A9" s="12"/>
+      <x:c r="A9" s="3"/>
       <x:c r="B9" s="12"/>
-      <x:c r="C9" s="12"/>
-      <x:c r="D9" s="3"/>
+      <x:c r="C9" s="3"/>
+      <x:c r="D9" s="12"/>
       <x:c r="E9" s="3"/>
       <x:c r="F9" s="3"/>
       <x:c r="G9" s="3"/>
-      <x:c r="H9" s="15"/>
+      <x:c r="H9" s="3"/>
       <x:c r="I9" s="3"/>
       <x:c r="J9" s="3"/>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
-      <x:c r="A10" s="12"/>
+      <x:c r="A10" s="10"/>
       <x:c r="B10" s="12"/>
-      <x:c r="C10" s="12"/>
-      <x:c r="D10" s="10"/>
+      <x:c r="C10" s="10"/>
+      <x:c r="D10" s="12"/>
       <x:c r="E10" s="10"/>
       <x:c r="F10" s="10"/>
       <x:c r="G10" s="10"/>
-      <x:c r="H10" s="14"/>
+      <x:c r="H10" s="10"/>
       <x:c r="I10" s="10"/>
       <x:c r="J10" s="10"/>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
-      <x:c r="A11" s="12"/>
+      <x:c r="A11" s="3"/>
       <x:c r="B11" s="12"/>
-      <x:c r="C11" s="12"/>
-      <x:c r="D11" s="3"/>
+      <x:c r="C11" s="3"/>
+      <x:c r="D11" s="12"/>
       <x:c r="E11" s="3"/>
       <x:c r="F11" s="3"/>
       <x:c r="G11" s="3"/>
-      <x:c r="H11" s="15"/>
+      <x:c r="H11" s="3"/>
       <x:c r="I11" s="3"/>
       <x:c r="J11" s="3"/>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
-      <x:c r="A12" s="12"/>
+      <x:c r="A12" s="10"/>
       <x:c r="B12" s="12"/>
-      <x:c r="C12" s="12"/>
-      <x:c r="D12" s="10"/>
+      <x:c r="C12" s="10"/>
+      <x:c r="D12" s="12"/>
       <x:c r="E12" s="10"/>
       <x:c r="F12" s="10"/>
       <x:c r="G12" s="10"/>
-      <x:c r="H12" s="14"/>
+      <x:c r="H12" s="10"/>
       <x:c r="I12" s="10"/>
       <x:c r="J12" s="10"/>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
-      <x:c r="A13" s="12"/>
+      <x:c r="A13" s="3"/>
       <x:c r="B13" s="12"/>
-      <x:c r="C13" s="12"/>
-      <x:c r="D13" s="3"/>
+      <x:c r="C13" s="3"/>
+      <x:c r="D13" s="12"/>
       <x:c r="E13" s="3"/>
       <x:c r="F13" s="3"/>
       <x:c r="G13" s="3"/>
-      <x:c r="H13" s="15"/>
+      <x:c r="H13" s="3"/>
       <x:c r="I13" s="3"/>
       <x:c r="J13" s="3"/>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
-      <x:c r="A14" s="12"/>
+      <x:c r="A14" s="10"/>
       <x:c r="B14" s="12"/>
-      <x:c r="C14" s="12"/>
-      <x:c r="D14" s="10"/>
+      <x:c r="C14" s="10"/>
+      <x:c r="D14" s="12"/>
       <x:c r="E14" s="10"/>
       <x:c r="F14" s="10"/>
       <x:c r="G14" s="10"/>
-      <x:c r="H14" s="14"/>
+      <x:c r="H14" s="10"/>
       <x:c r="I14" s="10"/>
       <x:c r="J14" s="10"/>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
-      <x:c r="A15" s="12"/>
+      <x:c r="A15" s="3"/>
       <x:c r="B15" s="12"/>
-      <x:c r="C15" s="12"/>
-      <x:c r="D15" s="3"/>
+      <x:c r="C15" s="3"/>
+      <x:c r="D15" s="12"/>
       <x:c r="E15" s="3"/>
       <x:c r="F15" s="3"/>
       <x:c r="G15" s="3"/>
-      <x:c r="H15" s="15"/>
+      <x:c r="H15" s="3"/>
       <x:c r="I15" s="3"/>
       <x:c r="J15" s="3"/>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
-      <x:c r="A16" s="12"/>
+      <x:c r="A16" s="10"/>
       <x:c r="B16" s="12"/>
-      <x:c r="C16" s="12"/>
-      <x:c r="D16" s="10"/>
+      <x:c r="C16" s="10"/>
+      <x:c r="D16" s="12"/>
       <x:c r="E16" s="10"/>
       <x:c r="F16" s="10"/>
       <x:c r="G16" s="10"/>
-      <x:c r="H16" s="14"/>
+      <x:c r="H16" s="10"/>
       <x:c r="I16" s="10"/>
       <x:c r="J16" s="10"/>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
-      <x:c r="A17" s="12"/>
+      <x:c r="A17" s="3"/>
       <x:c r="B17" s="12"/>
-      <x:c r="C17" s="12"/>
-      <x:c r="D17" s="3"/>
+      <x:c r="C17" s="3"/>
+      <x:c r="D17" s="12"/>
       <x:c r="E17" s="3"/>
       <x:c r="F17" s="3"/>
       <x:c r="G17" s="3"/>
-      <x:c r="H17" s="15"/>
+      <x:c r="H17" s="3"/>
       <x:c r="I17" s="3"/>
       <x:c r="J17" s="3"/>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
-      <x:c r="A18" s="12"/>
+      <x:c r="A18" s="10"/>
       <x:c r="B18" s="12"/>
-      <x:c r="C18" s="12"/>
-      <x:c r="D18" s="10"/>
+      <x:c r="C18" s="10"/>
+      <x:c r="D18" s="12"/>
       <x:c r="E18" s="10"/>
       <x:c r="F18" s="10"/>
       <x:c r="G18" s="10"/>
-      <x:c r="H18" s="14"/>
+      <x:c r="H18" s="10"/>
       <x:c r="I18" s="10"/>
       <x:c r="J18" s="10"/>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
-      <x:c r="A19" s="12"/>
+      <x:c r="A19" s="3"/>
       <x:c r="B19" s="12"/>
-      <x:c r="C19" s="12"/>
-      <x:c r="D19" s="3"/>
+      <x:c r="C19" s="3"/>
+      <x:c r="D19" s="12"/>
       <x:c r="E19" s="3"/>
       <x:c r="F19" s="3"/>
       <x:c r="G19" s="3"/>
-      <x:c r="H19" s="15"/>
+      <x:c r="H19" s="3"/>
       <x:c r="I19" s="3"/>
       <x:c r="J19" s="3"/>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
-      <x:c r="A20" s="12"/>
+      <x:c r="A20" s="10"/>
       <x:c r="B20" s="12"/>
-      <x:c r="C20" s="12"/>
-      <x:c r="D20" s="10"/>
+      <x:c r="C20" s="10"/>
+      <x:c r="D20" s="12"/>
       <x:c r="E20" s="10"/>
       <x:c r="F20" s="10"/>
       <x:c r="G20" s="10"/>
-      <x:c r="H20" s="14"/>
+      <x:c r="H20" s="10"/>
       <x:c r="I20" s="10"/>
       <x:c r="J20" s="10"/>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
-      <x:c r="A21" s="12"/>
+      <x:c r="A21" s="3"/>
       <x:c r="B21" s="12"/>
-      <x:c r="C21" s="12"/>
-      <x:c r="D21" s="3"/>
+      <x:c r="C21" s="3"/>
+      <x:c r="D21" s="12"/>
       <x:c r="E21" s="3"/>
       <x:c r="F21" s="3"/>
       <x:c r="G21" s="3"/>
-      <x:c r="H21" s="15"/>
+      <x:c r="H21" s="3"/>
       <x:c r="I21" s="3"/>
       <x:c r="J21" s="3"/>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
-      <x:c r="A22" s="12"/>
+      <x:c r="A22" s="10"/>
       <x:c r="B22" s="12"/>
-      <x:c r="C22" s="12"/>
-      <x:c r="D22" s="10"/>
+      <x:c r="C22" s="10"/>
+      <x:c r="D22" s="12"/>
       <x:c r="E22" s="10"/>
       <x:c r="F22" s="10"/>
       <x:c r="G22" s="10"/>
-      <x:c r="H22" s="14"/>
+      <x:c r="H22" s="10"/>
       <x:c r="I22" s="10"/>
       <x:c r="J22" s="10"/>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
-      <x:c r="A23" s="12"/>
+      <x:c r="A23" s="3"/>
       <x:c r="B23" s="12"/>
-      <x:c r="C23" s="12"/>
-      <x:c r="D23" s="3"/>
+      <x:c r="C23" s="3"/>
+      <x:c r="D23" s="12"/>
       <x:c r="E23" s="3"/>
       <x:c r="F23" s="3"/>
       <x:c r="G23" s="3"/>
-      <x:c r="H23" s="15"/>
+      <x:c r="H23" s="3"/>
       <x:c r="I23" s="3"/>
       <x:c r="J23" s="3"/>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
-      <x:c r="A24" s="12"/>
+      <x:c r="A24" s="10"/>
       <x:c r="B24" s="12"/>
-      <x:c r="C24" s="12"/>
-      <x:c r="D24" s="10"/>
+      <x:c r="C24" s="10"/>
+      <x:c r="D24" s="12"/>
       <x:c r="E24" s="10"/>
       <x:c r="F24" s="10"/>
       <x:c r="G24" s="10"/>
-      <x:c r="H24" s="14"/>
+      <x:c r="H24" s="10"/>
       <x:c r="I24" s="10"/>
       <x:c r="J24" s="10"/>
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
-      <x:c r="A25" s="12"/>
+      <x:c r="A25" s="3"/>
       <x:c r="B25" s="12"/>
-      <x:c r="C25" s="12"/>
-      <x:c r="D25" s="3"/>
+      <x:c r="C25" s="3"/>
+      <x:c r="D25" s="12"/>
       <x:c r="E25" s="3"/>
       <x:c r="F25" s="3"/>
       <x:c r="G25" s="3"/>
-      <x:c r="H25" s="15"/>
+      <x:c r="H25" s="3"/>
       <x:c r="I25" s="3"/>
       <x:c r="J25" s="3"/>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
-      <x:c r="A26" s="12"/>
+      <x:c r="A26" s="10"/>
       <x:c r="B26" s="12"/>
-      <x:c r="C26" s="12"/>
-      <x:c r="D26" s="10"/>
+      <x:c r="C26" s="10"/>
+      <x:c r="D26" s="12"/>
       <x:c r="E26" s="10"/>
       <x:c r="F26" s="10"/>
       <x:c r="G26" s="10"/>
-      <x:c r="H26" s="14"/>
+      <x:c r="H26" s="10"/>
       <x:c r="I26" s="10"/>
       <x:c r="J26" s="10"/>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
-      <x:c r="A27" s="12"/>
+      <x:c r="A27" s="3"/>
       <x:c r="B27" s="12"/>
-      <x:c r="C27" s="12"/>
-      <x:c r="D27" s="3"/>
+      <x:c r="C27" s="3"/>
+      <x:c r="D27" s="12"/>
       <x:c r="E27" s="3"/>
       <x:c r="F27" s="3"/>
       <x:c r="G27" s="3"/>
-      <x:c r="H27" s="15"/>
+      <x:c r="H27" s="3"/>
       <x:c r="I27" s="3"/>
       <x:c r="J27" s="3"/>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
-      <x:c r="A28" s="12"/>
+      <x:c r="A28" s="10"/>
       <x:c r="B28" s="12"/>
-      <x:c r="C28" s="12"/>
-      <x:c r="D28" s="10"/>
+      <x:c r="C28" s="10"/>
+      <x:c r="D28" s="12"/>
       <x:c r="E28" s="10"/>
       <x:c r="F28" s="10"/>
       <x:c r="G28" s="10"/>
-      <x:c r="H28" s="14"/>
+      <x:c r="H28" s="10"/>
       <x:c r="I28" s="10"/>
       <x:c r="J28" s="10"/>
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
-      <x:c r="A29" s="12"/>
+      <x:c r="A29" s="3"/>
       <x:c r="B29" s="12"/>
-      <x:c r="C29" s="12"/>
-      <x:c r="D29" s="3"/>
+      <x:c r="C29" s="3"/>
+      <x:c r="D29" s="12"/>
       <x:c r="E29" s="3"/>
       <x:c r="F29" s="3"/>
       <x:c r="G29" s="3"/>
-      <x:c r="H29" s="15"/>
+      <x:c r="H29" s="3"/>
       <x:c r="I29" s="3"/>
       <x:c r="J29" s="3"/>
     </x:row>
     <x:row r="30" ht="25" customHeight="1">
-      <x:c r="A30" s="12"/>
+      <x:c r="A30" s="10"/>
       <x:c r="B30" s="12"/>
-      <x:c r="C30" s="12"/>
-      <x:c r="D30" s="10"/>
+      <x:c r="C30" s="10"/>
+      <x:c r="D30" s="12"/>
       <x:c r="E30" s="10"/>
       <x:c r="F30" s="10"/>
       <x:c r="G30" s="10"/>
-      <x:c r="H30" s="14"/>
+      <x:c r="H30" s="10"/>
       <x:c r="I30" s="10"/>
       <x:c r="J30" s="10"/>
     </x:row>
     <x:row r="31" ht="25" customHeight="1">
-      <x:c r="A31" s="12"/>
+      <x:c r="A31" s="3"/>
       <x:c r="B31" s="12"/>
-      <x:c r="C31" s="12"/>
-      <x:c r="D31" s="3"/>
+      <x:c r="C31" s="3"/>
+      <x:c r="D31" s="12"/>
       <x:c r="E31" s="3"/>
       <x:c r="F31" s="3"/>
       <x:c r="G31" s="3"/>
-      <x:c r="H31" s="15"/>
+      <x:c r="H31" s="3"/>
       <x:c r="I31" s="3"/>
       <x:c r="J31" s="3"/>
     </x:row>
     <x:row r="32" ht="25" customHeight="1">
-      <x:c r="A32" s="12"/>
+      <x:c r="A32" s="10"/>
       <x:c r="B32" s="12"/>
-      <x:c r="C32" s="12"/>
-      <x:c r="D32" s="10"/>
+      <x:c r="C32" s="10"/>
+      <x:c r="D32" s="12"/>
       <x:c r="E32" s="10"/>
       <x:c r="F32" s="10"/>
       <x:c r="G32" s="10"/>
-      <x:c r="H32" s="14"/>
+      <x:c r="H32" s="10"/>
       <x:c r="I32" s="10"/>
       <x:c r="J32" s="10"/>
     </x:row>
     <x:row r="33" ht="25" customHeight="1">
-      <x:c r="A33" s="12"/>
+      <x:c r="A33" s="3"/>
       <x:c r="B33" s="12"/>
-      <x:c r="C33" s="12"/>
-      <x:c r="D33" s="3"/>
+      <x:c r="C33" s="3"/>
+      <x:c r="D33" s="12"/>
       <x:c r="E33" s="3"/>
       <x:c r="F33" s="3"/>
       <x:c r="G33" s="3"/>
-      <x:c r="H33" s="15"/>
+      <x:c r="H33" s="3"/>
       <x:c r="I33" s="3"/>
       <x:c r="J33" s="3"/>
     </x:row>
     <x:row r="34" ht="25" customHeight="1">
-      <x:c r="A34" s="12"/>
+      <x:c r="A34" s="10"/>
       <x:c r="B34" s="12"/>
-      <x:c r="C34" s="12"/>
-      <x:c r="D34" s="10"/>
+      <x:c r="C34" s="10"/>
+      <x:c r="D34" s="12"/>
       <x:c r="E34" s="10"/>
       <x:c r="F34" s="10"/>
       <x:c r="G34" s="10"/>
-      <x:c r="H34" s="14"/>
+      <x:c r="H34" s="10"/>
       <x:c r="I34" s="10"/>
       <x:c r="J34" s="10"/>
     </x:row>
     <x:row r="35" ht="25" customHeight="1">
-      <x:c r="A35" s="12"/>
+      <x:c r="A35" s="3"/>
       <x:c r="B35" s="12"/>
-      <x:c r="C35" s="12"/>
-      <x:c r="D35" s="3"/>
+      <x:c r="C35" s="3"/>
+      <x:c r="D35" s="12"/>
       <x:c r="E35" s="3"/>
       <x:c r="F35" s="3"/>
       <x:c r="G35" s="3"/>
-      <x:c r="H35" s="15"/>
+      <x:c r="H35" s="3"/>
       <x:c r="I35" s="3"/>
       <x:c r="J35" s="3"/>
     </x:row>
     <x:row r="36" ht="25" customHeight="1">
-      <x:c r="A36" s="12"/>
+      <x:c r="A36" s="10"/>
       <x:c r="B36" s="12"/>
-      <x:c r="C36" s="12"/>
-      <x:c r="D36" s="10"/>
+      <x:c r="C36" s="10"/>
+      <x:c r="D36" s="12"/>
       <x:c r="E36" s="10"/>
       <x:c r="F36" s="10"/>
       <x:c r="G36" s="10"/>
-      <x:c r="H36" s="14"/>
+      <x:c r="H36" s="10"/>
       <x:c r="I36" s="10"/>
       <x:c r="J36" s="10"/>
     </x:row>
     <x:row r="37" ht="25" customHeight="1">
-      <x:c r="A37" s="12"/>
+      <x:c r="A37" s="3"/>
       <x:c r="B37" s="12"/>
-      <x:c r="C37" s="12"/>
-      <x:c r="D37" s="3"/>
+      <x:c r="C37" s="3"/>
+      <x:c r="D37" s="12"/>
       <x:c r="E37" s="3"/>
       <x:c r="F37" s="3"/>
       <x:c r="G37" s="3"/>
-      <x:c r="H37" s="15"/>
+      <x:c r="H37" s="3"/>
       <x:c r="I37" s="3"/>
       <x:c r="J37" s="3"/>
     </x:row>
     <x:row r="38" ht="25" customHeight="1">
-      <x:c r="A38" s="12"/>
+      <x:c r="A38" s="10"/>
       <x:c r="B38" s="12"/>
-      <x:c r="C38" s="12"/>
-      <x:c r="D38" s="10"/>
+      <x:c r="C38" s="10"/>
+      <x:c r="D38" s="12"/>
       <x:c r="E38" s="10"/>
       <x:c r="F38" s="10"/>
       <x:c r="G38" s="10"/>
-      <x:c r="H38" s="14"/>
+      <x:c r="H38" s="10"/>
       <x:c r="I38" s="10"/>
       <x:c r="J38" s="10"/>
     </x:row>
     <x:row r="39" ht="25" customHeight="1">
-      <x:c r="A39" s="12"/>
+      <x:c r="A39" s="3"/>
       <x:c r="B39" s="12"/>
-      <x:c r="C39" s="12"/>
-      <x:c r="D39" s="3"/>
+      <x:c r="C39" s="3"/>
+      <x:c r="D39" s="12"/>
       <x:c r="E39" s="3"/>
       <x:c r="F39" s="3"/>
       <x:c r="G39" s="3"/>
-      <x:c r="H39" s="15"/>
+      <x:c r="H39" s="3"/>
       <x:c r="I39" s="3"/>
       <x:c r="J39" s="3"/>
     </x:row>
     <x:row r="40" ht="25" customHeight="1">
-      <x:c r="A40" s="12"/>
+      <x:c r="A40" s="10"/>
       <x:c r="B40" s="12"/>
-      <x:c r="C40" s="12"/>
-      <x:c r="D40" s="10"/>
+      <x:c r="C40" s="10"/>
+      <x:c r="D40" s="12"/>
       <x:c r="E40" s="10"/>
       <x:c r="F40" s="10"/>
       <x:c r="G40" s="10"/>
-      <x:c r="H40" s="14"/>
+      <x:c r="H40" s="10"/>
       <x:c r="I40" s="10"/>
       <x:c r="J40" s="10"/>
     </x:row>
     <x:row r="41" ht="25" customHeight="1">
-      <x:c r="A41" s="12"/>
+      <x:c r="A41" s="3"/>
       <x:c r="B41" s="12"/>
-      <x:c r="C41" s="12"/>
-      <x:c r="D41" s="3"/>
+      <x:c r="C41" s="3"/>
+      <x:c r="D41" s="12"/>
       <x:c r="E41" s="3"/>
       <x:c r="F41" s="3"/>
       <x:c r="G41" s="3"/>
-      <x:c r="H41" s="15"/>
+      <x:c r="H41" s="3"/>
       <x:c r="I41" s="3"/>
       <x:c r="J41" s="3"/>
     </x:row>
     <x:row r="42" ht="25" customHeight="1">
-      <x:c r="A42" s="12"/>
+      <x:c r="A42" s="10"/>
       <x:c r="B42" s="12"/>
-      <x:c r="C42" s="12"/>
-      <x:c r="D42" s="10"/>
+      <x:c r="C42" s="10"/>
+      <x:c r="D42" s="12"/>
       <x:c r="E42" s="10"/>
       <x:c r="F42" s="10"/>
       <x:c r="G42" s="10"/>
-      <x:c r="H42" s="14"/>
+      <x:c r="H42" s="10"/>
       <x:c r="I42" s="10"/>
       <x:c r="J42" s="10"/>
     </x:row>
     <x:row r="43" ht="25" customHeight="1">
-      <x:c r="A43" s="12"/>
+      <x:c r="A43" s="3"/>
       <x:c r="B43" s="12"/>
-      <x:c r="C43" s="12"/>
-      <x:c r="D43" s="3"/>
+      <x:c r="C43" s="3"/>
+      <x:c r="D43" s="12"/>
       <x:c r="E43" s="3"/>
       <x:c r="F43" s="3"/>
       <x:c r="G43" s="3"/>
-      <x:c r="H43" s="15"/>
+      <x:c r="H43" s="3"/>
       <x:c r="I43" s="3"/>
       <x:c r="J43" s="3"/>
     </x:row>
     <x:row r="44" ht="25" customHeight="1">
-      <x:c r="A44" s="12"/>
+      <x:c r="A44" s="10"/>
       <x:c r="B44" s="12"/>
-      <x:c r="C44" s="12"/>
-      <x:c r="D44" s="10"/>
+      <x:c r="C44" s="10"/>
+      <x:c r="D44" s="12"/>
       <x:c r="E44" s="10"/>
       <x:c r="F44" s="10"/>
       <x:c r="G44" s="10"/>
-      <x:c r="H44" s="14"/>
+      <x:c r="H44" s="10"/>
       <x:c r="I44" s="10"/>
       <x:c r="J44" s="10"/>
     </x:row>
     <x:row r="45" ht="25" customHeight="1">
-      <x:c r="A45" s="12"/>
+      <x:c r="A45" s="3"/>
       <x:c r="B45" s="12"/>
-      <x:c r="C45" s="12"/>
-      <x:c r="D45" s="3"/>
+      <x:c r="C45" s="3"/>
+      <x:c r="D45" s="12"/>
       <x:c r="E45" s="3"/>
       <x:c r="F45" s="3"/>
       <x:c r="G45" s="3"/>
-      <x:c r="H45" s="15"/>
+      <x:c r="H45" s="3"/>
       <x:c r="I45" s="3"/>
       <x:c r="J45" s="3"/>
     </x:row>
     <x:row r="46" ht="25" customHeight="1">
-      <x:c r="A46" s="12"/>
+      <x:c r="A46" s="10"/>
       <x:c r="B46" s="12"/>
-      <x:c r="C46" s="12"/>
-      <x:c r="D46" s="10"/>
+      <x:c r="C46" s="10"/>
+      <x:c r="D46" s="12"/>
       <x:c r="E46" s="10"/>
       <x:c r="F46" s="10"/>
       <x:c r="G46" s="10"/>
-      <x:c r="H46" s="14"/>
+      <x:c r="H46" s="10"/>
       <x:c r="I46" s="10"/>
       <x:c r="J46" s="10"/>
     </x:row>
     <x:row r="47" ht="25" customHeight="1">
-      <x:c r="A47" s="12"/>
+      <x:c r="A47" s="3"/>
       <x:c r="B47" s="12"/>
-      <x:c r="C47" s="12"/>
-      <x:c r="D47" s="3"/>
+      <x:c r="C47" s="3"/>
+      <x:c r="D47" s="12"/>
       <x:c r="E47" s="3"/>
       <x:c r="F47" s="3"/>
       <x:c r="G47" s="3"/>
-      <x:c r="H47" s="15"/>
+      <x:c r="H47" s="3"/>
       <x:c r="I47" s="3"/>
       <x:c r="J47" s="3"/>
     </x:row>
     <x:row r="48" ht="25" customHeight="1">
-      <x:c r="A48" s="12"/>
+      <x:c r="A48" s="10"/>
       <x:c r="B48" s="12"/>
-      <x:c r="C48" s="12"/>
-      <x:c r="D48" s="10"/>
+      <x:c r="C48" s="10"/>
+      <x:c r="D48" s="12"/>
       <x:c r="E48" s="10"/>
       <x:c r="F48" s="10"/>
       <x:c r="G48" s="10"/>
-      <x:c r="H48" s="14"/>
+      <x:c r="H48" s="10"/>
       <x:c r="I48" s="10"/>
       <x:c r="J48" s="10"/>
     </x:row>
     <x:row r="49" ht="25" customHeight="1">
-      <x:c r="A49" s="12"/>
+      <x:c r="A49" s="3"/>
       <x:c r="B49" s="12"/>
-      <x:c r="C49" s="12"/>
-      <x:c r="D49" s="3"/>
+      <x:c r="C49" s="3"/>
+      <x:c r="D49" s="12"/>
       <x:c r="E49" s="3"/>
       <x:c r="F49" s="3"/>
       <x:c r="G49" s="3"/>
-      <x:c r="H49" s="15"/>
+      <x:c r="H49" s="3"/>
       <x:c r="I49" s="3"/>
       <x:c r="J49" s="3"/>
     </x:row>
     <x:row r="50" ht="25" customHeight="1">
-      <x:c r="A50" s="12"/>
+      <x:c r="A50" s="10"/>
       <x:c r="B50" s="12"/>
-      <x:c r="C50" s="12"/>
-      <x:c r="D50" s="10"/>
+      <x:c r="C50" s="10"/>
+      <x:c r="D50" s="12"/>
       <x:c r="E50" s="10"/>
       <x:c r="F50" s="10"/>
       <x:c r="G50" s="10"/>
-      <x:c r="H50" s="14"/>
+      <x:c r="H50" s="10"/>
       <x:c r="I50" s="10"/>
       <x:c r="J50" s="10"/>
     </x:row>
     <x:row r="51" ht="25" customHeight="1">
-      <x:c r="A51" s="12"/>
+      <x:c r="A51" s="3"/>
       <x:c r="B51" s="12"/>
-      <x:c r="C51" s="12"/>
-      <x:c r="D51" s="3"/>
+      <x:c r="C51" s="3"/>
+      <x:c r="D51" s="12"/>
       <x:c r="E51" s="3"/>
       <x:c r="F51" s="3"/>
       <x:c r="G51" s="3"/>
-      <x:c r="H51" s="15"/>
+      <x:c r="H51" s="3"/>
       <x:c r="I51" s="3"/>
       <x:c r="J51" s="3"/>
     </x:row>
     <x:row r="52" ht="25" customHeight="1">
-      <x:c r="A52" s="12"/>
+      <x:c r="A52" s="10"/>
       <x:c r="B52" s="12"/>
-      <x:c r="C52" s="12"/>
-      <x:c r="D52" s="10"/>
+      <x:c r="C52" s="10"/>
+      <x:c r="D52" s="12"/>
       <x:c r="E52" s="10"/>
       <x:c r="F52" s="10"/>
       <x:c r="G52" s="10"/>
-      <x:c r="H52" s="14"/>
+      <x:c r="H52" s="10"/>
       <x:c r="I52" s="10"/>
       <x:c r="J52" s="10"/>
     </x:row>
     <x:row r="53" ht="25" customHeight="1">
-      <x:c r="A53" s="12"/>
+      <x:c r="A53" s="3"/>
       <x:c r="B53" s="12"/>
-      <x:c r="C53" s="12"/>
-      <x:c r="D53" s="3"/>
+      <x:c r="C53" s="3"/>
+      <x:c r="D53" s="12"/>
       <x:c r="E53" s="3"/>
       <x:c r="F53" s="3"/>
       <x:c r="G53" s="3"/>
-      <x:c r="H53" s="15"/>
+      <x:c r="H53" s="3"/>
       <x:c r="I53" s="3"/>
       <x:c r="J53" s="3"/>
     </x:row>
     <x:row r="54" ht="25" customHeight="1">
-      <x:c r="A54" s="12"/>
+      <x:c r="A54" s="10"/>
       <x:c r="B54" s="12"/>
-      <x:c r="C54" s="12"/>
-      <x:c r="D54" s="10"/>
+      <x:c r="C54" s="10"/>
+      <x:c r="D54" s="12"/>
       <x:c r="E54" s="10"/>
       <x:c r="F54" s="10"/>
       <x:c r="G54" s="10"/>
-      <x:c r="H54" s="14"/>
+      <x:c r="H54" s="10"/>
       <x:c r="I54" s="10"/>
       <x:c r="J54" s="10"/>
     </x:row>
     <x:row r="55" ht="25" customHeight="1">
-      <x:c r="A55" s="12"/>
+      <x:c r="A55" s="3"/>
       <x:c r="B55" s="12"/>
-      <x:c r="C55" s="12"/>
-      <x:c r="D55" s="3"/>
+      <x:c r="C55" s="3"/>
+      <x:c r="D55" s="12"/>
       <x:c r="E55" s="3"/>
       <x:c r="F55" s="3"/>
       <x:c r="G55" s="3"/>
-      <x:c r="H55" s="15"/>
+      <x:c r="H55" s="3"/>
       <x:c r="I55" s="3"/>
       <x:c r="J55" s="3"/>
     </x:row>
     <x:row r="56" ht="25" customHeight="1">
-      <x:c r="A56" s="12"/>
+      <x:c r="A56" s="10"/>
       <x:c r="B56" s="12"/>
-      <x:c r="C56" s="12"/>
-      <x:c r="D56" s="10"/>
+      <x:c r="C56" s="10"/>
+      <x:c r="D56" s="12"/>
       <x:c r="E56" s="10"/>
       <x:c r="F56" s="10"/>
       <x:c r="G56" s="10"/>
-      <x:c r="H56" s="14"/>
+      <x:c r="H56" s="10"/>
       <x:c r="I56" s="10"/>
       <x:c r="J56" s="10"/>
     </x:row>
     <x:row r="57" ht="25" customHeight="1">
-      <x:c r="A57" s="12"/>
+      <x:c r="A57" s="3"/>
       <x:c r="B57" s="12"/>
-      <x:c r="C57" s="12"/>
-      <x:c r="D57" s="3"/>
+      <x:c r="C57" s="3"/>
+      <x:c r="D57" s="12"/>
       <x:c r="E57" s="3"/>
       <x:c r="F57" s="3"/>
       <x:c r="G57" s="3"/>
-      <x:c r="H57" s="15"/>
+      <x:c r="H57" s="3"/>
       <x:c r="I57" s="3"/>
       <x:c r="J57" s="3"/>
     </x:row>
     <x:row r="58" ht="25" customHeight="1">
-      <x:c r="A58" s="12"/>
+      <x:c r="A58" s="10"/>
       <x:c r="B58" s="12"/>
-      <x:c r="C58" s="12"/>
-      <x:c r="D58" s="10"/>
+      <x:c r="C58" s="10"/>
+      <x:c r="D58" s="12"/>
       <x:c r="E58" s="10"/>
       <x:c r="F58" s="10"/>
       <x:c r="G58" s="10"/>
-      <x:c r="H58" s="14"/>
+      <x:c r="H58" s="10"/>
       <x:c r="I58" s="10"/>
       <x:c r="J58" s="10"/>
     </x:row>
     <x:row r="59" ht="25" customHeight="1">
-      <x:c r="A59" s="12"/>
+      <x:c r="A59" s="3"/>
       <x:c r="B59" s="12"/>
-      <x:c r="C59" s="12"/>
-      <x:c r="D59" s="3"/>
+      <x:c r="C59" s="3"/>
+      <x:c r="D59" s="12"/>
       <x:c r="E59" s="3"/>
       <x:c r="F59" s="3"/>
       <x:c r="G59" s="3"/>
-      <x:c r="H59" s="15"/>
+      <x:c r="H59" s="3"/>
       <x:c r="I59" s="3"/>
       <x:c r="J59" s="3"/>
     </x:row>
     <x:row r="60" ht="25" customHeight="1">
-      <x:c r="A60" s="12"/>
+      <x:c r="A60" s="10"/>
       <x:c r="B60" s="12"/>
-      <x:c r="C60" s="12"/>
-      <x:c r="D60" s="10"/>
+      <x:c r="C60" s="10"/>
+      <x:c r="D60" s="12"/>
       <x:c r="E60" s="10"/>
       <x:c r="F60" s="10"/>
       <x:c r="G60" s="10"/>
-      <x:c r="H60" s="14"/>
+      <x:c r="H60" s="10"/>
       <x:c r="I60" s="10"/>
       <x:c r="J60" s="10"/>
     </x:row>
     <x:row r="61" ht="25" customHeight="1">
-      <x:c r="A61" s="12"/>
+      <x:c r="A61" s="3"/>
       <x:c r="B61" s="12"/>
-      <x:c r="C61" s="12"/>
-      <x:c r="D61" s="3"/>
+      <x:c r="C61" s="3"/>
+      <x:c r="D61" s="12"/>
       <x:c r="E61" s="3"/>
       <x:c r="F61" s="3"/>
       <x:c r="G61" s="3"/>
-      <x:c r="H61" s="15"/>
+      <x:c r="H61" s="3"/>
       <x:c r="I61" s="3"/>
       <x:c r="J61" s="3"/>
     </x:row>
     <x:row r="62" ht="25" customHeight="1">
-      <x:c r="A62" s="12"/>
+      <x:c r="A62" s="10"/>
       <x:c r="B62" s="12"/>
-      <x:c r="C62" s="12"/>
-      <x:c r="D62" s="10"/>
+      <x:c r="C62" s="10"/>
+      <x:c r="D62" s="12"/>
       <x:c r="E62" s="10"/>
       <x:c r="F62" s="10"/>
       <x:c r="G62" s="10"/>
-      <x:c r="H62" s="14"/>
+      <x:c r="H62" s="10"/>
       <x:c r="I62" s="10"/>
       <x:c r="J62" s="10"/>
     </x:row>
     <x:row r="63" ht="25" customHeight="1">
-      <x:c r="A63" s="12"/>
+      <x:c r="A63" s="3"/>
       <x:c r="B63" s="12"/>
-      <x:c r="C63" s="12"/>
-      <x:c r="D63" s="3"/>
+      <x:c r="C63" s="3"/>
+      <x:c r="D63" s="12"/>
       <x:c r="E63" s="3"/>
       <x:c r="F63" s="3"/>
       <x:c r="G63" s="3"/>
-      <x:c r="H63" s="15"/>
+      <x:c r="H63" s="3"/>
       <x:c r="I63" s="3"/>
       <x:c r="J63" s="3"/>
     </x:row>
     <x:row r="64" ht="25" customHeight="1">
-      <x:c r="A64" s="12"/>
+      <x:c r="A64" s="10"/>
       <x:c r="B64" s="12"/>
-      <x:c r="C64" s="12"/>
-      <x:c r="D64" s="10"/>
+      <x:c r="C64" s="10"/>
+      <x:c r="D64" s="12"/>
       <x:c r="E64" s="10"/>
       <x:c r="F64" s="10"/>
       <x:c r="G64" s="10"/>
-      <x:c r="H64" s="14"/>
+      <x:c r="H64" s="10"/>
       <x:c r="I64" s="10"/>
       <x:c r="J64" s="10"/>
     </x:row>
     <x:row r="65" ht="25" customHeight="1">
-      <x:c r="A65" s="12"/>
+      <x:c r="A65" s="3"/>
       <x:c r="B65" s="12"/>
-      <x:c r="C65" s="12"/>
-      <x:c r="D65" s="3"/>
+      <x:c r="C65" s="3"/>
+      <x:c r="D65" s="12"/>
       <x:c r="E65" s="3"/>
       <x:c r="F65" s="3"/>
       <x:c r="G65" s="3"/>
-      <x:c r="H65" s="15"/>
+      <x:c r="H65" s="3"/>
       <x:c r="I65" s="3"/>
       <x:c r="J65" s="3"/>
     </x:row>
     <x:row r="66" ht="25" customHeight="1">
-      <x:c r="A66" s="12"/>
+      <x:c r="A66" s="10"/>
       <x:c r="B66" s="12"/>
-      <x:c r="C66" s="12"/>
-      <x:c r="D66" s="10"/>
+      <x:c r="C66" s="10"/>
+      <x:c r="D66" s="12"/>
       <x:c r="E66" s="10"/>
       <x:c r="F66" s="10"/>
       <x:c r="G66" s="10"/>
-      <x:c r="H66" s="14"/>
+      <x:c r="H66" s="10"/>
       <x:c r="I66" s="10"/>
       <x:c r="J66" s="10"/>
     </x:row>
     <x:row r="67" ht="25" customHeight="1">
-      <x:c r="A67" s="12"/>
+      <x:c r="A67" s="3"/>
       <x:c r="B67" s="12"/>
-      <x:c r="C67" s="12"/>
-      <x:c r="D67" s="3"/>
+      <x:c r="C67" s="3"/>
+      <x:c r="D67" s="12"/>
       <x:c r="E67" s="3"/>
       <x:c r="F67" s="3"/>
       <x:c r="G67" s="3"/>
-      <x:c r="H67" s="15"/>
+      <x:c r="H67" s="3"/>
       <x:c r="I67" s="3"/>
       <x:c r="J67" s="3"/>
     </x:row>
     <x:row r="68" ht="25" customHeight="1">
-      <x:c r="A68" s="12"/>
+      <x:c r="A68" s="10"/>
       <x:c r="B68" s="12"/>
-      <x:c r="C68" s="12"/>
-      <x:c r="D68" s="10"/>
+      <x:c r="C68" s="10"/>
+      <x:c r="D68" s="12"/>
       <x:c r="E68" s="10"/>
       <x:c r="F68" s="10"/>
       <x:c r="G68" s="10"/>
-      <x:c r="H68" s="14"/>
+      <x:c r="H68" s="10"/>
       <x:c r="I68" s="10"/>
       <x:c r="J68" s="10"/>
     </x:row>
     <x:row r="69" ht="25" customHeight="1">
-      <x:c r="A69" s="12"/>
+      <x:c r="A69" s="3"/>
       <x:c r="B69" s="12"/>
-      <x:c r="C69" s="12"/>
-      <x:c r="D69" s="3"/>
+      <x:c r="C69" s="3"/>
+      <x:c r="D69" s="12"/>
       <x:c r="E69" s="3"/>
       <x:c r="F69" s="3"/>
       <x:c r="G69" s="3"/>
-      <x:c r="H69" s="15"/>
+      <x:c r="H69" s="3"/>
       <x:c r="I69" s="3"/>
       <x:c r="J69" s="3"/>
     </x:row>
     <x:row r="70" ht="25" customHeight="1">
-      <x:c r="A70" s="12"/>
+      <x:c r="A70" s="10"/>
       <x:c r="B70" s="12"/>
-      <x:c r="C70" s="12"/>
-      <x:c r="D70" s="10"/>
+      <x:c r="C70" s="10"/>
+      <x:c r="D70" s="12"/>
       <x:c r="E70" s="10"/>
       <x:c r="F70" s="10"/>
       <x:c r="G70" s="10"/>
-      <x:c r="H70" s="14"/>
+      <x:c r="H70" s="10"/>
       <x:c r="I70" s="10"/>
       <x:c r="J70" s="10"/>
     </x:row>
     <x:row r="71" ht="25" customHeight="1">
-      <x:c r="A71" s="12"/>
+      <x:c r="A71" s="3"/>
       <x:c r="B71" s="12"/>
-      <x:c r="C71" s="12"/>
-      <x:c r="D71" s="3"/>
+      <x:c r="C71" s="3"/>
+      <x:c r="D71" s="12"/>
       <x:c r="E71" s="3"/>
       <x:c r="F71" s="3"/>
       <x:c r="G71" s="3"/>
-      <x:c r="H71" s="15"/>
+      <x:c r="H71" s="3"/>
       <x:c r="I71" s="3"/>
       <x:c r="J71" s="3"/>
     </x:row>
     <x:row r="72" ht="25" customHeight="1">
-      <x:c r="A72" s="12"/>
+      <x:c r="A72" s="10"/>
       <x:c r="B72" s="12"/>
-      <x:c r="C72" s="12"/>
-      <x:c r="D72" s="10"/>
+      <x:c r="C72" s="10"/>
+      <x:c r="D72" s="12"/>
       <x:c r="E72" s="10"/>
       <x:c r="F72" s="10"/>
       <x:c r="G72" s="10"/>
-      <x:c r="H72" s="14"/>
+      <x:c r="H72" s="10"/>
       <x:c r="I72" s="10"/>
       <x:c r="J72" s="10"/>
     </x:row>
     <x:row r="73" ht="25" customHeight="1">
-      <x:c r="A73" s="12"/>
+      <x:c r="A73" s="3"/>
       <x:c r="B73" s="12"/>
-      <x:c r="C73" s="12"/>
-      <x:c r="D73" s="3"/>
+      <x:c r="C73" s="3"/>
+      <x:c r="D73" s="12"/>
       <x:c r="E73" s="3"/>
       <x:c r="F73" s="3"/>
       <x:c r="G73" s="3"/>
-      <x:c r="H73" s="15"/>
+      <x:c r="H73" s="3"/>
       <x:c r="I73" s="3"/>
       <x:c r="J73" s="3"/>
     </x:row>
     <x:row r="74" ht="25" customHeight="1">
-      <x:c r="A74" s="12"/>
+      <x:c r="A74" s="10"/>
       <x:c r="B74" s="12"/>
-      <x:c r="C74" s="12"/>
-      <x:c r="D74" s="10"/>
+      <x:c r="C74" s="10"/>
+      <x:c r="D74" s="12"/>
       <x:c r="E74" s="10"/>
       <x:c r="F74" s="10"/>
       <x:c r="G74" s="10"/>
-      <x:c r="H74" s="14"/>
+      <x:c r="H74" s="10"/>
       <x:c r="I74" s="10"/>
       <x:c r="J74" s="10"/>
     </x:row>
     <x:row r="75" ht="25" customHeight="1">
-      <x:c r="A75" s="12"/>
+      <x:c r="A75" s="3"/>
       <x:c r="B75" s="12"/>
-      <x:c r="C75" s="12"/>
-      <x:c r="D75" s="3"/>
+      <x:c r="C75" s="3"/>
+      <x:c r="D75" s="12"/>
       <x:c r="E75" s="3"/>
       <x:c r="F75" s="3"/>
       <x:c r="G75" s="3"/>
-      <x:c r="H75" s="15"/>
+      <x:c r="H75" s="3"/>
       <x:c r="I75" s="3"/>
       <x:c r="J75" s="3"/>
     </x:row>
     <x:row r="76" ht="25" customHeight="1">
-      <x:c r="A76" s="12"/>
+      <x:c r="A76" s="10"/>
       <x:c r="B76" s="12"/>
-      <x:c r="C76" s="12"/>
-      <x:c r="D76" s="10"/>
+      <x:c r="C76" s="10"/>
+      <x:c r="D76" s="12"/>
       <x:c r="E76" s="10"/>
       <x:c r="F76" s="10"/>
       <x:c r="G76" s="10"/>
-      <x:c r="H76" s="14"/>
+      <x:c r="H76" s="10"/>
       <x:c r="I76" s="10"/>
       <x:c r="J76" s="10"/>
     </x:row>
     <x:row r="77" ht="25" customHeight="1">
-      <x:c r="A77" s="12"/>
+      <x:c r="A77" s="3"/>
       <x:c r="B77" s="12"/>
-      <x:c r="C77" s="12"/>
-      <x:c r="D77" s="3"/>
+      <x:c r="C77" s="3"/>
+      <x:c r="D77" s="12"/>
       <x:c r="E77" s="3"/>
       <x:c r="F77" s="3"/>
       <x:c r="G77" s="3"/>
-      <x:c r="H77" s="15"/>
+      <x:c r="H77" s="3"/>
       <x:c r="I77" s="3"/>
       <x:c r="J77" s="3"/>
     </x:row>
     <x:row r="78" ht="25" customHeight="1">
-      <x:c r="A78" s="12"/>
+      <x:c r="A78" s="10"/>
       <x:c r="B78" s="12"/>
-      <x:c r="C78" s="12"/>
-      <x:c r="D78" s="10"/>
+      <x:c r="C78" s="10"/>
+      <x:c r="D78" s="12"/>
       <x:c r="E78" s="10"/>
       <x:c r="F78" s="10"/>
       <x:c r="G78" s="10"/>
-      <x:c r="H78" s="14"/>
+      <x:c r="H78" s="10"/>
       <x:c r="I78" s="10"/>
       <x:c r="J78" s="10"/>
     </x:row>
     <x:row r="79" ht="25" customHeight="1">
-      <x:c r="A79" s="12"/>
+      <x:c r="A79" s="3"/>
       <x:c r="B79" s="12"/>
-      <x:c r="C79" s="12"/>
-      <x:c r="D79" s="3"/>
+      <x:c r="C79" s="3"/>
+      <x:c r="D79" s="12"/>
       <x:c r="E79" s="3"/>
       <x:c r="F79" s="3"/>
       <x:c r="G79" s="3"/>
-      <x:c r="H79" s="15"/>
+      <x:c r="H79" s="3"/>
       <x:c r="I79" s="3"/>
       <x:c r="J79" s="3"/>
     </x:row>
     <x:row r="80" ht="25" customHeight="1">
-      <x:c r="A80" s="12"/>
+      <x:c r="A80" s="10"/>
       <x:c r="B80" s="12"/>
-      <x:c r="C80" s="12"/>
-      <x:c r="D80" s="10"/>
+      <x:c r="C80" s="10"/>
+      <x:c r="D80" s="12"/>
       <x:c r="E80" s="10"/>
       <x:c r="F80" s="10"/>
       <x:c r="G80" s="10"/>
-      <x:c r="H80" s="14"/>
+      <x:c r="H80" s="10"/>
       <x:c r="I80" s="10"/>
       <x:c r="J80" s="10"/>
     </x:row>
     <x:row r="81" ht="25" customHeight="1">
-      <x:c r="A81" s="12"/>
+      <x:c r="A81" s="3"/>
       <x:c r="B81" s="12"/>
-      <x:c r="C81" s="12"/>
-      <x:c r="D81" s="3"/>
+      <x:c r="C81" s="3"/>
+      <x:c r="D81" s="12"/>
       <x:c r="E81" s="3"/>
       <x:c r="F81" s="3"/>
       <x:c r="G81" s="3"/>
-      <x:c r="H81" s="15"/>
+      <x:c r="H81" s="3"/>
       <x:c r="I81" s="3"/>
       <x:c r="J81" s="3"/>
     </x:row>
     <x:row r="82" ht="25" customHeight="1">
-      <x:c r="A82" s="12"/>
+      <x:c r="A82" s="10"/>
       <x:c r="B82" s="12"/>
-      <x:c r="C82" s="12"/>
-      <x:c r="D82" s="10"/>
+      <x:c r="C82" s="10"/>
+      <x:c r="D82" s="12"/>
       <x:c r="E82" s="10"/>
       <x:c r="F82" s="10"/>
       <x:c r="G82" s="10"/>
-      <x:c r="H82" s="14"/>
+      <x:c r="H82" s="10"/>
       <x:c r="I82" s="10"/>
       <x:c r="J82" s="10"/>
     </x:row>
     <x:row r="83" ht="25" customHeight="1">
-      <x:c r="A83" s="12"/>
+      <x:c r="A83" s="3"/>
       <x:c r="B83" s="12"/>
-      <x:c r="C83" s="12"/>
-      <x:c r="D83" s="3"/>
+      <x:c r="C83" s="3"/>
+      <x:c r="D83" s="12"/>
       <x:c r="E83" s="3"/>
       <x:c r="F83" s="3"/>
       <x:c r="G83" s="3"/>
-      <x:c r="H83" s="15"/>
+      <x:c r="H83" s="3"/>
       <x:c r="I83" s="3"/>
       <x:c r="J83" s="3"/>
     </x:row>
     <x:row r="84" ht="25" customHeight="1">
-      <x:c r="A84" s="12"/>
+      <x:c r="A84" s="10"/>
       <x:c r="B84" s="12"/>
-      <x:c r="C84" s="12"/>
-      <x:c r="D84" s="10"/>
+      <x:c r="C84" s="10"/>
+      <x:c r="D84" s="12"/>
       <x:c r="E84" s="10"/>
       <x:c r="F84" s="10"/>
       <x:c r="G84" s="10"/>
-      <x:c r="H84" s="14"/>
+      <x:c r="H84" s="10"/>
       <x:c r="I84" s="10"/>
       <x:c r="J84" s="10"/>
     </x:row>
     <x:row r="85" ht="25" customHeight="1">
-      <x:c r="A85" s="12"/>
+      <x:c r="A85" s="3"/>
       <x:c r="B85" s="12"/>
-      <x:c r="C85" s="12"/>
-      <x:c r="D85" s="3"/>
+      <x:c r="C85" s="3"/>
+      <x:c r="D85" s="12"/>
       <x:c r="E85" s="3"/>
       <x:c r="F85" s="3"/>
       <x:c r="G85" s="3"/>
-      <x:c r="H85" s="15"/>
+      <x:c r="H85" s="3"/>
       <x:c r="I85" s="3"/>
       <x:c r="J85" s="3"/>
     </x:row>
     <x:row r="86" ht="25" customHeight="1">
-      <x:c r="A86" s="12"/>
+      <x:c r="A86" s="10"/>
       <x:c r="B86" s="12"/>
-      <x:c r="C86" s="12"/>
-      <x:c r="D86" s="10"/>
+      <x:c r="C86" s="10"/>
+      <x:c r="D86" s="12"/>
       <x:c r="E86" s="10"/>
       <x:c r="F86" s="10"/>
       <x:c r="G86" s="10"/>
-      <x:c r="H86" s="14"/>
+      <x:c r="H86" s="10"/>
       <x:c r="I86" s="10"/>
       <x:c r="J86" s="10"/>
     </x:row>
     <x:row r="87" ht="25" customHeight="1">
-      <x:c r="A87" s="12"/>
+      <x:c r="A87" s="3"/>
       <x:c r="B87" s="12"/>
-      <x:c r="C87" s="12"/>
-      <x:c r="D87" s="3"/>
+      <x:c r="C87" s="3"/>
+      <x:c r="D87" s="12"/>
       <x:c r="E87" s="3"/>
       <x:c r="F87" s="3"/>
       <x:c r="G87" s="3"/>
-      <x:c r="H87" s="15"/>
+      <x:c r="H87" s="3"/>
       <x:c r="I87" s="3"/>
       <x:c r="J87" s="3"/>
     </x:row>
     <x:row r="88" ht="25" customHeight="1">
-      <x:c r="A88" s="12"/>
+      <x:c r="A88" s="10"/>
       <x:c r="B88" s="12"/>
-      <x:c r="C88" s="12"/>
-      <x:c r="D88" s="10"/>
+      <x:c r="C88" s="10"/>
+      <x:c r="D88" s="12"/>
       <x:c r="E88" s="10"/>
       <x:c r="F88" s="10"/>
       <x:c r="G88" s="10"/>
-      <x:c r="H88" s="14"/>
+      <x:c r="H88" s="10"/>
       <x:c r="I88" s="10"/>
       <x:c r="J88" s="10"/>
     </x:row>
     <x:row r="89" ht="25" customHeight="1">
-      <x:c r="A89" s="12"/>
+      <x:c r="A89" s="3"/>
       <x:c r="B89" s="12"/>
-      <x:c r="C89" s="12"/>
-      <x:c r="D89" s="3"/>
+      <x:c r="C89" s="3"/>
+      <x:c r="D89" s="12"/>
       <x:c r="E89" s="3"/>
       <x:c r="F89" s="3"/>
       <x:c r="G89" s="3"/>
-      <x:c r="H89" s="15"/>
+      <x:c r="H89" s="3"/>
       <x:c r="I89" s="3"/>
       <x:c r="J89" s="3"/>
     </x:row>
     <x:row r="90" ht="25" customHeight="1">
-      <x:c r="A90" s="12"/>
+      <x:c r="A90" s="10"/>
       <x:c r="B90" s="12"/>
-      <x:c r="C90" s="12"/>
-      <x:c r="D90" s="10"/>
+      <x:c r="C90" s="10"/>
+      <x:c r="D90" s="12"/>
       <x:c r="E90" s="10"/>
       <x:c r="F90" s="10"/>
       <x:c r="G90" s="10"/>
-      <x:c r="H90" s="14"/>
+      <x:c r="H90" s="10"/>
       <x:c r="I90" s="10"/>
       <x:c r="J90" s="10"/>
     </x:row>
     <x:row r="91" ht="25" customHeight="1">
-      <x:c r="A91" s="12"/>
+      <x:c r="A91" s="3"/>
       <x:c r="B91" s="12"/>
-      <x:c r="C91" s="12"/>
-      <x:c r="D91" s="3"/>
+      <x:c r="C91" s="3"/>
+      <x:c r="D91" s="12"/>
       <x:c r="E91" s="3"/>
       <x:c r="F91" s="3"/>
       <x:c r="G91" s="3"/>
-      <x:c r="H91" s="15"/>
+      <x:c r="H91" s="3"/>
       <x:c r="I91" s="3"/>
       <x:c r="J91" s="3"/>
     </x:row>
     <x:row r="92" ht="25" customHeight="1">
-      <x:c r="A92" s="12"/>
+      <x:c r="A92" s="10"/>
       <x:c r="B92" s="12"/>
-      <x:c r="C92" s="12"/>
-      <x:c r="D92" s="10"/>
+      <x:c r="C92" s="10"/>
+      <x:c r="D92" s="12"/>
       <x:c r="E92" s="10"/>
       <x:c r="F92" s="10"/>
       <x:c r="G92" s="10"/>
-      <x:c r="H92" s="14"/>
+      <x:c r="H92" s="10"/>
       <x:c r="I92" s="10"/>
       <x:c r="J92" s="10"/>
     </x:row>
     <x:row r="93" ht="25" customHeight="1">
-      <x:c r="A93" s="12"/>
+      <x:c r="A93" s="3"/>
       <x:c r="B93" s="12"/>
-      <x:c r="C93" s="12"/>
-      <x:c r="D93" s="3"/>
+      <x:c r="C93" s="3"/>
+      <x:c r="D93" s="12"/>
       <x:c r="E93" s="3"/>
       <x:c r="F93" s="3"/>
       <x:c r="G93" s="3"/>
-      <x:c r="H93" s="15"/>
+      <x:c r="H93" s="3"/>
       <x:c r="I93" s="3"/>
       <x:c r="J93" s="3"/>
     </x:row>
     <x:row r="94" ht="25" customHeight="1">
-      <x:c r="A94" s="12"/>
+      <x:c r="A94" s="10"/>
       <x:c r="B94" s="12"/>
-      <x:c r="C94" s="12"/>
-      <x:c r="D94" s="10"/>
+      <x:c r="C94" s="10"/>
+      <x:c r="D94" s="12"/>
       <x:c r="E94" s="10"/>
       <x:c r="F94" s="10"/>
       <x:c r="G94" s="10"/>
-      <x:c r="H94" s="14"/>
+      <x:c r="H94" s="10"/>
       <x:c r="I94" s="10"/>
       <x:c r="J94" s="10"/>
     </x:row>
     <x:row r="95" ht="25" customHeight="1">
-      <x:c r="A95" s="12"/>
+      <x:c r="A95" s="3"/>
       <x:c r="B95" s="12"/>
-      <x:c r="C95" s="12"/>
-      <x:c r="D95" s="3"/>
+      <x:c r="C95" s="3"/>
+      <x:c r="D95" s="12"/>
       <x:c r="E95" s="3"/>
       <x:c r="F95" s="3"/>
       <x:c r="G95" s="3"/>
-      <x:c r="H95" s="15"/>
+      <x:c r="H95" s="3"/>
       <x:c r="I95" s="3"/>
       <x:c r="J95" s="3"/>
     </x:row>
     <x:row r="96" ht="25" customHeight="1">
-      <x:c r="A96" s="12"/>
+      <x:c r="A96" s="10"/>
       <x:c r="B96" s="12"/>
-      <x:c r="C96" s="12"/>
-      <x:c r="D96" s="10"/>
+      <x:c r="C96" s="10"/>
+      <x:c r="D96" s="12"/>
       <x:c r="E96" s="10"/>
       <x:c r="F96" s="10"/>
       <x:c r="G96" s="10"/>
-      <x:c r="H96" s="14"/>
+      <x:c r="H96" s="10"/>
       <x:c r="I96" s="10"/>
       <x:c r="J96" s="10"/>
     </x:row>
     <x:row r="97" ht="25" customHeight="1">
-      <x:c r="A97" s="12"/>
+      <x:c r="A97" s="3"/>
       <x:c r="B97" s="12"/>
-      <x:c r="C97" s="12"/>
-      <x:c r="D97" s="3"/>
+      <x:c r="C97" s="3"/>
+      <x:c r="D97" s="12"/>
       <x:c r="E97" s="3"/>
       <x:c r="F97" s="3"/>
       <x:c r="G97" s="3"/>
-      <x:c r="H97" s="15"/>
+      <x:c r="H97" s="3"/>
       <x:c r="I97" s="3"/>
       <x:c r="J97" s="3"/>
     </x:row>
     <x:row r="98" ht="25" customHeight="1">
-      <x:c r="A98" s="12"/>
+      <x:c r="A98" s="10"/>
       <x:c r="B98" s="12"/>
-      <x:c r="C98" s="12"/>
-      <x:c r="D98" s="10"/>
+      <x:c r="C98" s="10"/>
+      <x:c r="D98" s="12"/>
       <x:c r="E98" s="10"/>
       <x:c r="F98" s="10"/>
       <x:c r="G98" s="10"/>
-      <x:c r="H98" s="14"/>
+      <x:c r="H98" s="10"/>
       <x:c r="I98" s="10"/>
       <x:c r="J98" s="10"/>
     </x:row>
     <x:row r="99" ht="25" customHeight="1">
-      <x:c r="A99" s="12"/>
+      <x:c r="A99" s="3"/>
       <x:c r="B99" s="12"/>
-      <x:c r="C99" s="12"/>
-      <x:c r="D99" s="3"/>
+      <x:c r="C99" s="3"/>
+      <x:c r="D99" s="12"/>
       <x:c r="E99" s="3"/>
       <x:c r="F99" s="3"/>
       <x:c r="G99" s="3"/>
-      <x:c r="H99" s="15"/>
+      <x:c r="H99" s="3"/>
       <x:c r="I99" s="3"/>
       <x:c r="J99" s="3"/>
     </x:row>
     <x:row r="100" ht="25" customHeight="1">
-      <x:c r="A100" s="12"/>
+      <x:c r="A100" s="10"/>
       <x:c r="B100" s="12"/>
-      <x:c r="C100" s="12"/>
-      <x:c r="D100" s="10"/>
+      <x:c r="C100" s="10"/>
+      <x:c r="D100" s="12"/>
       <x:c r="E100" s="10"/>
       <x:c r="F100" s="10"/>
       <x:c r="G100" s="10"/>
-      <x:c r="H100" s="14"/>
+      <x:c r="H100" s="10"/>
       <x:c r="I100" s="10"/>
       <x:c r="J100" s="10"/>
     </x:row>
     <x:row r="101" ht="25" customHeight="1">
-      <x:c r="A101" s="12"/>
+      <x:c r="A101" s="3"/>
       <x:c r="B101" s="12"/>
-      <x:c r="C101" s="12"/>
-      <x:c r="D101" s="3"/>
+      <x:c r="C101" s="3"/>
+      <x:c r="D101" s="12"/>
       <x:c r="E101" s="3"/>
       <x:c r="F101" s="3"/>
       <x:c r="G101" s="3"/>
-      <x:c r="H101" s="15"/>
+      <x:c r="H101" s="3"/>
       <x:c r="I101" s="3"/>
       <x:c r="J101" s="3"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="C2:C101">
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="D2:D101">
       <x:formula1>"Activo,Prospecto,Inactivo"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I2:I101">
-      <x:formula1>"Sí,No"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="H2:H101">
-      <x:formula1>1</x:formula1>
-      <x:formula2>31</x:formula2>
+    <x:dataValidation type="list" sqref="F2:F101">
+      <x:formula1>"Farmacéutica,Alimentos y bebidas,Logística y almacenamiento,Comercio y distribución,Manufactura,Construcción,Agricultura,Editorial e impresión,Servicios,Otros"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2330,10 +2319,10 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="35" customHeight="1">
-      <x:c r="A1" s="11" t="str">
+      <x:c r="A1" s="13" t="str">
         <x:v>referencia_cliente</x:v>
       </x:c>
-      <x:c r="B1" s="13" t="str">
+      <x:c r="B1" s="11" t="str">
         <x:v>nombre</x:v>
       </x:c>
       <x:c r="C1" s="8" t="str">
@@ -3176,10 +3165,10 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="35" customHeight="1">
-      <x:c r="A1" s="11" t="str">
+      <x:c r="A1" s="13" t="str">
         <x:v>referencia_cliente</x:v>
       </x:c>
-      <x:c r="B1" s="13" t="str">
+      <x:c r="B1" s="11" t="str">
         <x:v>nombre</x:v>
       </x:c>
       <x:c r="C1" s="8" t="str">

</xml_diff>

<commit_message>
Relaciona sedes con contactos del cliente y simplifica la captura
</commit_message>
<xml_diff>
--- a/public/templates/Plantilla-clientes-EMSA.xlsx
+++ b/public/templates/Plantilla-clientes-EMSA.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="1" r:id="Rb299d5d676c24288"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cliente" sheetId="2" r:id="R0a270c17b0ed4200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacto" sheetId="3" r:id="Ra75275d312ee4c75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sede" sheetId="4" r:id="R825c57e463c44a38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guía" sheetId="1" r:id="R57c06b764d984dbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cliente" sheetId="2" r:id="Ra80af6d4797a484d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacto" sheetId="3" r:id="Rdfcbef6596bc4789"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sede" sheetId="4" r:id="R7abc094f94c242f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -927,16 +927,16 @@
         <x:v>Sede</x:v>
       </x:c>
       <x:c r="B38" s="15" t="str">
-        <x:v>horario_atencion</x:v>
+        <x:v>referencia_ubicacion</x:v>
       </x:c>
       <x:c r="C38" s="15" t="str">
-        <x:v>Recomendado</x:v>
+        <x:v>Opcional</x:v>
       </x:c>
       <x:c r="D38" s="15" t="str">
-        <x:v>Días y horarios permitidos para servicios o visitas.</x:v>
+        <x:v>Plus Code o referencia para llegar a la sede.</x:v>
       </x:c>
       <x:c r="E38" s="15" t="str">
-        <x:v>Lunes a viernes de 8:00 a 17:00</x:v>
+        <x:v>Código y localidad</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="29" customHeight="1">
@@ -944,16 +944,16 @@
         <x:v>Sede</x:v>
       </x:c>
       <x:c r="B39" s="22" t="str">
-        <x:v>autoriza_ingreso</x:v>
+        <x:v>autoriza_contacto_id</x:v>
       </x:c>
       <x:c r="C39" s="22" t="str">
-        <x:v>Recomendado</x:v>
+        <x:v>Opcional</x:v>
       </x:c>
       <x:c r="D39" s="22" t="str">
-        <x:v>Persona o cargo que autoriza la entrada del técnico.</x:v>
+        <x:v>ID de contacto existente del mismo cliente; también puedes elegirlo después en la web.</x:v>
       </x:c>
       <x:c r="E39" s="22" t="str">
-        <x:v>Jefatura de mantenimiento</x:v>
+        <x:v>ID de una exportación</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="25" customHeight="1">
@@ -3181,10 +3181,10 @@
         <x:v>departamento</x:v>
       </x:c>
       <x:c r="F1" s="8" t="str">
-        <x:v>horario_atencion</x:v>
+        <x:v>referencia_ubicacion</x:v>
       </x:c>
       <x:c r="G1" s="9" t="str">
-        <x:v>autoriza_ingreso</x:v>
+        <x:v>autoriza_contacto_id</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">

</xml_diff>